<commit_message>
add more model options
</commit_message>
<xml_diff>
--- a/backend/audit_logs.xlsx
+++ b/backend/audit_logs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4845,6 +4845,258 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-01-04 22:37:07</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>gpt-5-nano-2025-08-07</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>df6192cb-a5ff-41f5-8e6b-979897bc5ced.pdf</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document f...</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document fragment.
+Input: The attached text from a contract.
+CRITICAL INSTRUCTIONS:
+1. **Assume Isolation with Common Sense**: Do NOT assume missing definitions exist in other documents. However, IGNORE common commercial lending terms typically defined in a base Credit Agreement (e.g., "Borrower", "Administrative Agent", "Lender", "Business Day", "Dollars", "GAAP", "Material Adverse Effect"). Only flag specific, deal-specific, or unusual capitalized terms that are undefined.
+2. **Logic Check:** Check all math and logic tables.
+3. **Drafting Errors:** Find any placeholders like "[__]" or blank lines that were forgotten.
+4. **Exact Quotes:** For every error, you MUST provide the `exact_quote` from the text that contains the error. This is used for highlighting.
+Output Format:
+Return ONLY a valid JSON object with the following structure:
+{
+  "errors": [
+    {
+      "location": "Page 3, Section 2.1",
+      "error": "Description of the error",
+      "suggestion": "Suggested fix",
+      "exact_quote": "Exact text substring to highlight in red"
+    }
+  ]
+}
+If no errors are found, return {"errors": []}.
+--- CONTRACT TEXT BEGINS ---
+--- [START OF PAGE 1] ---
+FIRST AMENDMENT TO AMENDED AND RESTATED
+CREDIT AGREEMENT
+This document is a generated test file containing intentional legal drafting errors for AI training
+purposes.
+ARTICLE I: DEFINITIONS
+...
+"Applicable Margin" means the corresponding percentages per annum as set forth below based on
+the Consolidated Total Leverage Ratio:
+Pricing Level
+Consolidated Total Leverage Ratio
+SOFR Margin
+I
+Greater than or equal to 3.25 to 1.00
+2.75%
+II
+Greater than or equal to 2.60 to 1.00 but less than 3.25 to 1.00
+2.50%
+III
+Greater than or equal to 1.75 to 1.00 but less than 2.50 to 1.00
+2.25%
+IV
+Greater than or equal to 1.50 to 1.00 but less than 1.75 to 1.00
+2.00%
+V
+Less than 1.50 to 1.00
+1.75%
+"Cash Collateral" shall have a meaning correlative to the foregoing and shall include the proceeds of
+such cash collateral...
+(Note: "Cash Collateralize" is defined, but "Cash Collateralization" is NOT defined
+in this section.)
+SECTION 2.5 Permanent Reduction of the Revolving Credit
+Commitment
+The Borrower shall have the right at any time to terminate the Revolving Credit Commitment...
+Any reduction of the Revolving Credit Commitment to zero shall be accompanied by payment of all
+outstanding Revolving Credit Loans and furnishing of Cash Collateralization satisfactory to the
+Administrative Agent.
+SECTION 5.13 Incremental Loans
+At any time after the First Amendment Effective Date, the Borrower may by written notice to the
+Administrative Agent elect to request the establishment of one or more increases in the Revolving
+--- [START OF PAGE 2] ---
+Credit Commitments...
+Such notice shall be delivered to the Administrative Agent at its office in [__] (or such other location as
+the Administrative Agent may designate).
+The terms of such Incremental Revolving Credit Increase shall be subject to the documentation
+requirements set forth in Section 5.19.
+[End of Document]
+--- CONTRACT TEXT ENDS ---</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>{
+  "errors": [
+    {
+      "location": "Page 1, Note under 'Cash Collateral' discussion (Definitions)",
+      "error": "Undefined term: 'Cash Collateralization' is not defined in this section although referenced elsewhere.",
+      "suggestion": "Define 'Cash Collateralization' with a clear meaning (or adjust references to 'Cash Collateralize' if that is the intended term).",
+      "exact_quote": "Note: \"Cash Collateralize\" is defined, but \"Cash Collateralization\" is NOT defined in this section."
+    },
+    {
+      "location": "Page 2, Section 5.13 Incremental Loans",
+      "error": "Placeholder missing: the notice delivery location is incomplete due to placeholder [__].",
+      "suggestion": "Fill in the office address or location for the Administrative Agent, e.g., \"Such notice shall be delivered to the Administrative Agent at its office in [insert address] (or such other location as the Administrative Agent may designate).\"",
+      "exact_quote": "Such notice shall be delivered to the Administrative Agent at its office in [__] (or such other location as the Administrative Agent may designate)."
+    },
+    {
+      "location": "Page 1, Section 5.13 Incremental Loans",
+      "error": "Drafting error / incomplete sentence: the sentence ends with an unfinished phrase; missing words after 'Revolving'.",
+      "suggestion": "Complete the sentence to read something like: \"... increases in the Revolving Credit Commitments\" (or the intended term) and ensure the section flows to Section 5.19 as referenced.",
+      "exact_quote": "At any time after the First Amendment Effective Date, the Borrower may by written notice to the Administrative Agent elect to request the establishment of one or more increases in the Revolving"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-01-04 22:38:40</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>gpt-5.2-2025-12-11</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>e5f73ce7-8a06-4dfc-9cf1-85286828df12.pdf</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document f...</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document fragment.
+Input: The attached text from a contract.
+CRITICAL INSTRUCTIONS:
+1. **Assume Isolation with Common Sense**: Do NOT assume missing definitions exist in other documents. However, IGNORE common commercial lending terms typically defined in a base Credit Agreement (e.g., "Borrower", "Administrative Agent", "Lender", "Business Day", "Dollars", "GAAP", "Material Adverse Effect"). Only flag specific, deal-specific, or unusual capitalized terms that are undefined.
+2. **Logic Check:** Check all math and logic tables.
+3. **Drafting Errors:** Find any placeholders like "[__]" or blank lines that were forgotten.
+4. **Exact Quotes:** For every error, you MUST provide the `exact_quote` from the text that contains the error. This is used for highlighting.
+Output Format:
+Return ONLY a valid JSON object with the following structure:
+{
+  "errors": [
+    {
+      "location": "Page 3, Section 2.1",
+      "error": "Description of the error",
+      "suggestion": "Suggested fix",
+      "exact_quote": "Exact text substring to highlight in red"
+    }
+  ]
+}
+If no errors are found, return {"errors": []}.
+--- CONTRACT TEXT BEGINS ---
+--- [START OF PAGE 1] ---
+FIRST AMENDMENT TO AMENDED AND RESTATED
+CREDIT AGREEMENT
+This document is a generated test file containing intentional legal drafting errors for AI training
+purposes.
+ARTICLE I: DEFINITIONS
+...
+"Applicable Margin" means the corresponding percentages per annum as set forth below based on
+the Consolidated Total Leverage Ratio:
+Pricing Level
+Consolidated Total Leverage Ratio
+SOFR Margin
+I
+Greater than or equal to 3.25 to 1.00
+2.75%
+II
+Greater than or equal to 2.60 to 1.00 but less than 3.25 to 1.00
+2.50%
+III
+Greater than or equal to 1.75 to 1.00 but less than 2.50 to 1.00
+2.25%
+IV
+Greater than or equal to 1.50 to 1.00 but less than 1.75 to 1.00
+2.00%
+V
+Less than 1.50 to 1.00
+1.75%
+"Cash Collateral" shall have a meaning correlative to the foregoing and shall include the proceeds of
+such cash collateral...
+(Note: "Cash Collateralize" is defined, but "Cash Collateralization" is NOT defined
+in this section.)
+SECTION 2.5 Permanent Reduction of the Revolving Credit
+Commitment
+The Borrower shall have the right at any time to terminate the Revolving Credit Commitment...
+Any reduction of the Revolving Credit Commitment to zero shall be accompanied by payment of all
+outstanding Revolving Credit Loans and furnishing of Cash Collateralization satisfactory to the
+Administrative Agent.
+SECTION 5.13 Incremental Loans
+At any time after the First Amendment Effective Date, the Borrower may by written notice to the
+Administrative Agent elect to request the establishment of one or more increases in the Revolving
+--- [START OF PAGE 2] ---
+Credit Commitments...
+Such notice shall be delivered to the Administrative Agent at its office in [__] (or such other location as
+the Administrative Agent may designate).
+The terms of such Incremental Revolving Credit Increase shall be subject to the documentation
+requirements set forth in Section 5.19.
+[End of Document]
+--- CONTRACT TEXT ENDS ---</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>{
+  "errors": [
+    {
+      "location": "Page 1, Article I (Definitions) – Applicable Margin table",
+      "error": "Logical gap/overlap risk in leverage ratio bands: Level I starts at “Greater than or equal to 3.25 to 1.00” while Level II ends at “less than 3.25 to 1.00.” This is generally fine, but the table does not expressly state whether the boundaries are intended to be inclusive/exclusive for each level in a consistent manner across all levels. As drafted, boundaries are inconsistently described (“greater than or equal to” vs. “less than”), which can create interpretive disputes at exact threshold values.",
+      "suggestion": "Revise the table to state the threshold logic consistently (e.g., make each band explicit as “≥ x and &lt; y” and state that Level I is “≥ 3.25,” Level V is “&lt; 1.50,” and all intermediate levels are “≥ lower and &lt; upper”).",
+      "exact_quote": "I\nGreater than or equal to 3.25 to 1.00\n2.75%\nII\nGreater than or equal to 2.60 to 1.00 but less than 3.25 to 1.00"
+    },
+    {
+      "location": "Page 1, Article I (Definitions) / Section 2.5",
+      "error": "Undefined (deal-specific/unusual) capitalized term used: “Cash Collateralization” is referenced but not defined. The text itself flags that “Cash Collateralize” is defined while “Cash Collateralization” is not, and the operative clause requires furnishing “Cash Collateralization” satisfactory to the Administrative Agent.",
+      "suggestion": "Either (a) add a definition of “Cash Collateralization” in the Definitions section (e.g., the act of Cash Collateralizing, and the required amount/forms), or (b) replace “Cash Collateralization” with the defined term “Cash Collateralize” (or other defined noun form), and adjust grammar accordingly.",
+      "exact_quote": "furnishing of Cash Collateralization satisfactory to the\nAdministrative Agent."
+    },
+    {
+      "location": "Page 2, Section 5.13 (Incremental Loans)",
+      "error": "Placeholder left in document: bracketed blank “[__]” for the Administrative Agent’s office location.",
+      "suggestion": "Replace “[__]” with the actual address/location (or remove and replace with a defined notice address concept consistent with the agreement’s notice provisions).",
+      "exact_quote": "Such notice shall be delivered to the Administrative Agent at its office in [__] (or such other location as\nthe Administrative Agent may designate)."
+    },
+    {
+      "location": "Page 2, Section 5.13 (Incremental Loans)",
+      "error": "Internal cross-reference appears incorrect or undefined in this fragment: “documentation requirements set forth in Section 5.19” is referenced, but Section 5.19 is not included/defined in the provided standalone fragment. Under the instruction to assume isolation (with common sense), this is an unresolved cross-reference.",
+      "suggestion": "If Section 5.19 exists in the underlying agreement, consider including it or adjusting the reference for this standalone document; otherwise, correct the section number to the intended section containing the documentation requirements.",
+      "exact_quote": "requirements set forth in Section 5.19."
+    }
+  ]
+}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update to glass style ui
</commit_message>
<xml_diff>
--- a/backend/audit_logs.xlsx
+++ b/backend/audit_logs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5097,6 +5097,722 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-01-05 22:35:01</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>gpt-5-nano-2025-08-07</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>a565ced2-30c5-43e5-9d87-bbef9f588693.pdf</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document f...</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document fragment.
+Input: The attached text from a contract.
+CRITICAL INSTRUCTIONS:
+1. **Assume Isolation with Common Sense**: Do NOT assume missing definitions exist in other documents. However, IGNORE common commercial lending terms typically defined in a base Credit Agreement (e.g., "Borrower", "Administrative Agent", "Lender", "Business Day", "Dollars", "GAAP", "Material Adverse Effect"). Only flag specific, deal-specific, or unusual capitalized terms that are undefined.
+2. **Logic Check:** Check all math and logic tables.
+3. **Drafting Errors:** Find any placeholders like "[__]" or blank lines that were forgotten.
+4. **Exact Quotes:** For every error, you MUST provide the `exact_quote` from the text that contains the error. This is used for highlighting.
+Output Format:
+Return ONLY a valid JSON object with the following structure:
+{
+  "errors": [
+    {
+      "location": "Page 3, Section 2.1",
+      "error": "Description of the error",
+      "suggestion": "Suggested fix",
+      "exact_quote": "Exact text substring to highlight in red"
+    }
+  ]
+}
+If no errors are found, return {"errors": []}.
+--- CONTRACT TEXT BEGINS ---
+--- [START OF PAGE 1] ---
+EX-10 2 tmb-20250626xex10.htm EX-10
+FIRST AMENDMENT TO AMENDED AND RESTATED CREDIT
+AGREEMENT
+FIRST AMENDMENT TO AMENDED AND RESTATED CREDIT AGREEMENT
+(this “Agreement”), dated as of June 26, 2025 (and effective as set forth below), among
+MAYVILLE ENGINEERING COMPANY, INC., a Wisconsin corporation (the “Borrower”),
+the Subsidiary Guarantors (as defined in the Existing Credit Agreement referred to below)
+party hereto, the Incremental Lenders (as defined below), the Lenders (as defined below)
+party hereto (the “Consenting Lenders”), and WELLS FARGO BANK, NATIONAL
+ASSOCIATION, as administrative agent (the “Administrative Agent”). Unless otherwise
+indicated, all capitalized terms used herein and not otherwise defined herein shall have the
+respective meanings provided such terms in the Credit Agreement referred to below.
+W I T N E S S E T H:
+WHEREAS, the Borrower, the lenders party thereto (the “Lenders”) and the
+Administrative Agent have entered into that certain Amended and Restated Credit Agreement,
+dated as of June 28, 2023 (as amended, restated, supplemented or otherwise modified prior to
+the date hereof, the “Existing Credit Agreement” and as hereby amended and as from time to
+time further amended, modified, supplemented, restated, or amended and restated, the “Credit
+Agreement”);
+WHEREAS, the Borrower has requested an Incremental Revolving Credit Increase in
+the aggregate principal amount of $100,000,000, in accordance with Section 5.13 of the
+Existing Credit Agreement (the “First Amendment Revolving Credit Increase”);
+WHEREAS, subject to the terms of this Agreement, certain of the Revolving Credit
+Lenders identified on the signature pages hereto (each an “Incremental Lender”) are severally
+willing to provide a portion of the First Amendment Revolving Credit Increase; and
+WHEREAS, the Borrower has also requested, and subject to the terms and conditions
+set forth herein, the Administrative Agent and the Consenting Lenders have agreed to further
+amend the Existing Credit Agreement as more specifically set forth herein.
+NOW, THEREFORE, in consideration of the foregoing and for other good and
+valuable consideration, the receipt and sufficiency of which are hereby acknowledged, it is
+agreed as follows:
+SECTION 1.Amendments to Existing Credit Agreement. Effective as of the First
+Amendment Effective Date (as defined below) and subject to the terms and conditions set
+forth herein and in reliance upon the representations and warranties set forth herein:
+(a)Schedule 1.1 (Commitments and Commitment Percentages) to the Existing
+Credit Agreement is hereby amended and restated in the form attached hereto
+as Annex A.
+(b)the body of Existing Credit Agreement is hereby amended as follows: (i) to
+delete red or green stricken text (indicated textually in the same manner as the
+following examples: stricken text and stricken text) and (ii) to add the blue or
+green double-underlined text (indicated textually in the same manner as the
+following examples: double-underlined text and double-underlined text), in
+each case, as set forth in the conformed copy attached hereto as Annex B.
+--- [START OF PAGE 2] ---
+1
+--- [START OF PAGE 3] ---
+SECTION 2.Revolving Credit Facility Increase; Reallocation.
+(a)Each Incremental Lender severally agrees that its Revolving Credit
+Commitment after giving effect to the First Amendment Revolving Credit
+Increase shall be as set forth opposite such Lender’s name on Annex A hereto.
+(b)The parties hereto hereby agree that (i) this Agreement constitutes a request
+for an Incremental Revolving Credit Increase pursuant to Section 5.13 of the
+Credit Agreement, (ii) the parties hereto hereby waive any prior notice
+required thereby, and (iii) this Agreement shall be deemed to be an “Lender
+Joinder Agreement” in accordance with Section 5.13(h) of the Credit
+Agreement.
+(c)Pursuant to Section 5.13 of the Credit Agreement, on the First Amendment
+Effective Date (as defined below) and after giving effect to this Agreement,
+the outstanding Revolving Credit Loans and Revolving Credit Commitment
+Percentages of Swingline Loans and L/C Obligations will be reallocated by
+the Administrative Agent among the Revolving Credit Lenders (including the
+Incremental Lenders providing the First Amendment Revolving Credit
+Increase) in accordance with their revised Revolving Credit Commitment
+Percentages (and the Revolving Credit Lenders (including the Incremental
+Lenders providing the First Amendment Revolving Credit Increase) agree to
+make all payments and adjustments necessary to effect such reallocation and
+the Borrower shall pay any and all costs required pursuant to Section 5.9 of
+the Credit Agreement in connection with such reallocation as if such
+reallocation were a repayment).
+SECTION 3.Conditions of Effectiveness of this Agreement.  This Agreement shall
+become effective on the date when the following conditions shall have been satisfied or
+waived (such date, the “First Amendment Effective Date”):
+(a) The Administrative Agent’s receipt of the following, each in form and
+substance reasonably satisfactory to the Administrative Agent:
+(i) this Agreement, duly executed by each of the Credit Parties existing
+as of the First Amendment Effective Date, the Administrative Agent, each
+Incremental Lender and each of the Consenting Lenders;
+(ii) a certificate of a Responsible Officer (or the secretary or assistant
+secretary) of each Credit Party certifying as to the incumbency and genuineness of the
+signature of each officer of such Credit Party executing Loan Documents to which it
+is a party and certifying that attached thereto is a true, correct and complete copy of
+(A) the articles or certificate of incorporation or formation (or equivalent), as
+applicable, of such Credit Party and all amendments thereto, certified as of a recent
+date by the appropriate Governmental Authority in its jurisdiction of incorporation,
+organization or formation (or equivalent), as applicable, (B) the bylaws or other
+governing document of such Credit Party as in effect on the First Amendment
+Effective Date, (C) resolutions duly adopted by the board of directors (or other
+governing body) of such Credit Party authorizing and approving the transactions
+contemplated hereunder and the execution, delivery and performance of this
+Amendment, the Credit Agreement and the other Loan Documents to which it is a
+party, and (D) certificates as of a recent date of the good standing of each Credit Party
+--- [START OF PAGE 4] ---
+2under the laws of its jurisdiction of incorporation, organization or formation (or
+equivalent), as applicable;
+(iii) an Officer’s Compliance Certificate demonstrating, in form and
+substance reasonably satisfactory to the Administrative Agent, that the Borrower is in
+compliance with the
+--- [START OF PAGE 5] ---
+financial covenants set forth in Section 9.15 of the Credit Agreement as of the First
+Amendment Effective Date based on the financial statements most recently delivered
+pursuant to Section 8.1(a) or 8.1(b) of the Existing Credit Agreement, as applicable,
+both before and after giving effect (on a pro forma basis) to (x) any Incremental
+Revolving Credit Commitment, and (y) the making of the First Amendment
+Revolving Credit Increase pursuant thereto (with such Incremental Revolving Credit
+Commitment being deemed to be fully funded);
+(iv) a certificate from the chief financial officer of the Borrower with
+respect to solvency (on a consolidated basis) of the Borrower and its Subsidiaries as
+of the First Amendment Effective Date after giving effect to the First Amendment
+Revolving Credit Increase and the other amendments contemplated by this
+Agreement;
+(v) an opinion from counsel to the Credit Parties, in form and substance
+reasonably satisfactory to the Administrative Agent.
+(b) The representations and warranties set forth in Section 3 shall be true and
+correct.
+(c) No Default or Event of Default shall exist on the First Amendment Effective
+Date immediately prior to or after giving effect to this Agreement.
+(d) The Administrative Agent shall have received the results of a Lien search, in
+form and substance reasonably satisfactory thereto, made against the Credit Parties under the
+Uniform Commercial Code (or applicable judicial docket) as in effect in each jurisdiction in
+which filings or recordations under the Uniform Commercial Code should be made to
+evidence or perfect security interests in all assets of such Credit Party, indicating among other
+things that the assets of each such Credit Party are free and clear of any Lien (except for
+Permitted Liens).
+(e) All governmental, shareholder and third party consents and approvals
+necessary (or any other material consents as determined in the reasonable discretion of the
+Administrative Agent) in connection with the transactions contemplated by this Agreement
+shall have been obtained and shall be in full force and effect.
+(f) The Borrower and each of the Subsidiary Guarantors shall have provided to
+the Administrative Agent and the Lenders, at least five (5) Business Days prior to the First
+Amendment Effective Date, a Beneficial Ownership Certification under 31 C.F.R. 1010.230
+and all documentation and other information required by regulatory authorities under
+applicable “know your customer”, anti-money-laundering, beneficial ownership and other
+similar rules and regulations, including, without limitation, the PATRIOT Act.
+(g) The Borrower shall have paid all fees and expenses required to be paid on the
+First Amendment Effective Date.
+For purposes of determining compliance with the conditions specified in this Section 3, the
+Administrative Agent, each Incremental Lender and each Consenting Lender that has signed
+this Agreement shall be deemed to have consented to, approved or accepted or to be satisfied
+with, each document or other matter required thereunder to be consented to or approved by or
+acceptable or satisfactory to an Incremental Lender and/or a Consenting Lender, as applicable,
+unless the Administrative Agent shall have received notice from such Incremental Lender
+--- [START OF PAGE 6] ---
+3and/or Consenting Lender, as applicable, prior to the proposed First Amendment Effective
+Date specifying its objection thereto.
+--- [START OF PAGE 7] ---
+SECTION 4.Representations and Warranties.  To induce the Administrative Agent,
+the Incremental Lenders party hereto and the Consenting Lenders party hereto to enter into
+this Agreement, each Credit Party represents and warrants to the Administrative Agent, the
+Incremental Lenders and the Consenting Lenders on and as of the First Amendment Effective
+Date that, in each case:
+(a) each of the representations and warranties contained in Article VII of the
+Credit Agreement are true and correct in all material respects, except to the extent any such
+representation and warranty is qualified by materiality or reference to Material Adverse
+Effect, in which case, such representation and warranty is true, correct and complete in all
+respects, with the same effect as if made on and as of such date (except for any such
+representation and warranty that by its terms is made only as of an earlier date, which
+representation and warranty remains true and correct as of such earlier date);
+(b) no Default or Event of Default has occurred and is continuing immediately
+prior to or after giving effect to this Agreement;
+(c) it has the right, power and authority and has taken all necessary corporate and
+other action to authorize the execution, delivery and performance of this Agreement in
+accordance with their respective terms; and
+(d) this Agreement has been duly executed and delivered by the duly authorized
+officers, managers, managing members or other authorized person of each Credit Party that is
+a party thereto, and each such document constitutes the legal, valid and binding obligation of
+each Credit Party, enforceable in accordance with its terms, except as such enforceability may
+be limited by bankruptcy, insolvency, reorganization, moratorium or similar state or federal
+Debtor Relief Laws from time to time in effect which affect the enforcement of creditors’
+rights in general and the availability of equitable remedies.
+SECTION 5.Credit Party Acknowledgements, Agreements and Confirmations.  By
+its execution of this Agreement, each Credit Party hereby (a) consents to this Agreement and
+agrees that the transactions contemplated by this Agreement shall not limit or diminish the
+obligations of such Credit Party, or release such Credit Party from any obligations, under any
+of the Loan Documents to which it is a party, (b) confirms and reaffirms its obligations under
+each of the Loan Documents to which it is a party and (c) agrees that each of the Loan
+Documents to which it is a party remain in full force and effect and are hereby ratified and
+confirmed.
+SECTION 6.Reference to and Effect on the Credit Agreement and the Loan
+Documents.
+(a) On and after the First Amendment Effective Date, each reference in the Credit
+Agreement to “this Agreement,” “herein,” “hereto”, “hereof” and “hereunder” or words of like
+import referring to the Credit Agreement, and each reference in the Notes and each of the
+other Loan Documents to “the Credit Agreement”, “thereunder”, “thereof” or words of like
+import referring to the Credit Agreement, shall mean and be a reference to the Credit
+Agreement, as amended and supplemented by this Agreement.
+(b) The Credit Agreement and each of the other Loan Documents, as specifically
+amended and supplemented by this Agreement, are and shall continue to be in full force and
+effect and are hereby in all respects ratified and confirmed.
+(c) The execution, delivery and effectiveness of this Agreement shall not, except
+as expressly provided herein, operate as a waiver of any right, power or remedy of any Lender
+or the Administrative Agent under any of the Loan Documents, nor constitute a waiver of any
+provision of any of the Loan Documents.  Without limiting the generality of the foregoing, the
+--- [START OF PAGE 8] ---
+4Security Documents in effect immediately prior to the date hereof and all of the Collateral
+described therein in existence immediately prior to the date hereof do and shall continue to
+secure the payment of all Secured Obligations.  
+--- [START OF PAGE 9] ---
+5(d) This Agreement is the entire agreement, and supersedes any prior agreements
+and contemporaneous oral agreements, of the parties concerning its subject matter. This
+Agreement shall constitute a “Loan Document” for all purposes of the Credit Agreement and
+the other Loan Documents.
+(e) This Agreement shall be binding on and inure to the benefit of the parties
+hereto and their successors and permitted assigns.
+SECTION 7.Costs and Expenses.  The Borrower hereby reconfirms its obligations
+pursuant to Section 12.3 of the Credit Agreement to pay and reimburse the Administrative
+Agent for all reasonable fees, costs and expenses in accordance with the terms thereof.
+SECTION 8.Governing Law; Jury Trial Waiver.  This Agreement and any claim,
+controversy, dispute or cause of action (whether in contract or tort or otherwise) based upon,
+arising out of or relating to this Agreement and the transactions contemplated hereby shall be
+governed by, and construed in accordance with, the law of the State of New York.  EACH
+PARTY HERETO HEREBY IRREVOCABLY WAIVES, TO THE FULLEST EXTENT
+PERMITTED BY APPLICABLE LAW, ANY RIGHT IT MAY HAVE TO A TRIAL BY JURY
+IN ANY LEGAL PROCEEDING DIRECTLY OR INDIRECTLY ARISING OUT OF OR
+RELATING TO THIS AGREEMENT OR THE TRANSACTIONS CONTEMPLATED
+HEREBY (WHETHER BASED ON CONTRACT, TORT OR ANY OTHER THEORY).  EACH
+PARTY HERETO (A) CERTIFIES THAT NO REPRESENTATIVE, AGENT OR ATTORNEY
+OF ANY OTHER PERSON HAS REPRESENTED, EXPRESSLY OR OTHERWISE, THAT
+SUCH OTHER PERSON WOULD NOT, IN THE EVENT OF LITIGATION, SEEK TO
+ENFORCE THE FOREGOING WAIVER AND (B) ACKNOWLEDGES THAT IT AND THE
+OTHER PARTIES HERETO HAVE BEEN INDUCED TO ENTER INTO THIS AGREEMENT
+BY, AMONG OTHER THINGS, THE MUTUAL WAIVERS AND CERTIFICATIONS IN THIS
+SECTION.
+SECTION 9.Counterparts; Electronic Execution. This Agreement may be executed
+in counterparts (and by different parties hereto in different counterparts), each of which shall
+constitute an original, but all of which when taken together shall constitute a single contract.
+Delivery of an executed counterpart of a signature page of this Agreement by facsimile or in
+electronic (i.e., “pdf” or “tif”) format shall be effective as delivery of a manually executed
+counterpart of this Agreement. This Agreement may be executed by Electronic Signatures or
+in the form of an Electronic Record pursuant to, and in accordance with, the provisions of
+Section 12.16 of the Credit Agreement.
+[Signature pages to follow]
+--- [START OF PAGE 10] ---
+Mayville Engineering Company, Inc.IN WITNESS WHEREOF, the parties hereto have caused their duly authorized
+officers to execute and deliver this Agreement as of the date first above written.
+BORROWER:
+MAYVILLE ENGINEERING COMPANY,
+INC.
+SUBSIDIARY GUARANTORS:
+CENTER MANUFACTURING
+HOLDINGS, INC.
+CENTER MANUFACTURING, INC.
+CENTER – MOELLER PRODUCTS LLC
+DEFIANCE METAL PRODUCTS CO.
+DEFIANCE METAL PRODUCTS OF
+ARKANSAS, INC. 
+ By:
+Name:
+Title:
+By:
+Name:
+Title:
+By:
+Name:
+Title:
+By:
+Name:
+Title:
+By:
+Name:
+Title:
+By:
+Name:
+Title:
+--- [START OF PAGE 11] ---
+First Amendment to A&amp;R Credit Agreement (Revolver Increase)
+Signature Page
+--- [START OF PAGE 12] ---
+Mayville Engineering Company, Inc.
+First Amendment to A&amp;R Credit Agreement (Revolver Increase)
+Signature PageDEFIANCE METAL PRODUCTS OF PA.,
+INC.
+MID-STATES ALUMINUM, LLC 
+ By:
+Name:
+Title:
+By:
+Name:
+Title:
+--- [START OF PAGE 13] ---
+Mayville Engineering Company, Inc.
+First Amendment to A&amp;R Credit Agreement (Revolver Increase)
+Signature PageWELLS FARGO BANK, NATIONAL
+ASSOCIATION, as Administrative Agent,
+Issuing Lender, Swingline Lender,
+Consenting Lender and an Incremental
+Lender
+By:
+___________________________________
+Name:
+Title:  
+--- [START OF PAGE 14] ---
+Mayville Engineering Company, Inc.
+First Amendment to A&amp;R Credit Agreement (Revolver Increase)
+Signature PageJPMORGAN CHASE BANK, N.A., as a
+Consenting Lender and an Incremental
+Lender
+By:
+___________________________________
+Name:
+Title:  
+--- [START OF PAGE 15] ---
+Mayville Engineering Company, Inc.
+First Amendment to A&amp;R Credit Agreement (Revolver Increase)
+Signature PageTD BANK, N.A., as a Consenting Lender
+and an Incremental Lender
+By:
+___________________________________
+Name:
+Title:  
+--- [START OF PAGE 16] ---
+Mayville Engineering Company, Inc.
+First Amendment to A&amp;R Credit Agreement (Revolver Increase)
+Signature PageCITIBANK, N.A., as a Consenting Lender
+By:
+___________________________________
+Name:
+Title:  
+--- [START OF PAGE 17] ---
+Mayville Engineering Company, Inc.
+First Amendment to A&amp;R Credit Agreement (Revolver Increase)
+Signature PageHANMI BANK, as a Consenting Lender and
+an Incremental Lender
+By:
+___________________________________
+Name:
+Title:  
+--- [START OF PAGE 18] ---
+Mayville Engineering Company, Inc.
+First Amendment to A&amp;R Credit Agreement (Revolver Increase)
+Signature PageASSOCIATED BANK, N.A., as a
+Consenting Lender and an Incremental
+Lender
+By:
+___________________________________
+Name:
+Title:  
+--- [START OF PAGE 19] ---
+Annex A
+REVOLVING CREDIT COMMITMENTS AND REVOLVING CREDIT COMMITMENT
+PERCENTAGES
+Lender Revolving
+Credit
+CommitmentRevolving
+Credit
+Commitment
+Percentage
+Wells Fargo Bank, National
+Association 
+$108,000,000.00 30.857142858%
+JPMorgan Chase Bank, N.A.  $90,000,000.00 25.714285714%
+TD Bank, N.A.  $77,000,000.00 22.000000000%
+Associated Bank, N.A.  $30,000,000.00 8.571428571%
+Hanmi Bank  $25,000,000.00 7.142857143%
+Citibank, N.A.  $20,000,000.00 5.714285714%
+Total $350,000,000.00100.000000000%
+--- [START OF PAGE 20] ---
+ANNEX B
+Published CUSIP Number: 57859VAP8
+$350,000,000.00
+AMENDED AND RESTATED CREDIT AGREEMENT
+dated as of June 28, 2023
+(as amended by that certain First Amendment to Amended and Restated Credit Agreement
+dated as of June 26, 2025)
+by and among
+MAYVILLE ENGINEERING COMPANY, INC.
+as Borrower,
+the Lenders referred to herein,
+as Lenders,
+and
+WELLS FARGO BANK, NATIONAL ASSOCIATION,
+as Administrative Agent,
+Swingline Lender and Issuing Lender
+and
+WELLS FARGO SECURITIES, LLC,
+as Joint Lead Arranger and Joint Bookrunner
+and
+J.P. MORGAN SECURITIES LLC,
+as Joint Lead Arranger and Joint Bookrunner
+and
+TD BANK, N.A.,
+as Joint Lead Arranger and Joint Bookrunner 
+--- [START OF PAGE 21] ---
+--- [START OF PAGE 22] ---
+i 
+ ARTICLE IDEFINITIONS 1
+SECTION 1.1Definitions 1
+SECTION 1.2Other Definitions and Provisions 31
+SECTION 1.3Accounting Terms 31
+SECTION 1.4UCC Terms 32
+SECTION 1.5Rounding 32
+SECTION 1.6References to Agreement and Laws 32
+SECTION 1.7Times of Day 32
+SECTION 1.8Letter of Credit Amounts 32
+SECTION 1.9Guarantees/Earn-Outs 33
+SECTION 1.10Covenant Compliance Generally 33
+SECTION 1.11Rates 33
+SECTION 1.12Divisions 33
+ARTICLE IIREVOLVING CREDIT FACILITY 34
+SECTION 2.1Revolving Credit Loans 34
+SECTION 2.2Swingline Loans 34
+SECTION 2.3Procedure for Advances of Revolving Credit Loans and Swingline
+Loans 36
+SECTION 2.4Repayment and Prepayment of Revolving Credit Loans and Swingline
+Loans 37
+SECTION 2.5Permanent Reduction of the Revolving Credit Commitment 37
+SECTION 2.6Termination of Revolving Credit Facility 38
+ARTICLE IIILETTER OF CREDIT FACILITY 38
+SECTION 3.1L/C Facility 38
+SECTION 3.2Procedure for Issuance of Letters of Credit 39
+SECTION 3.3Commissions and Other Charges 39
+SECTION 3.4L/C Participations 40
+SECTION 3.5Reimbursement Obligation of the Borrower 41
+SECTION 3.6Obligations Absolute 41
+SECTION 3.7Effect of Letter of Credit Application 41
+SECTION 3.8Resignation of Issuing Lenders 42
+SECTION 3.9Reporting of Letter of Credit Information and L/C Commitment 42
+SECTION 3.10Letters of Credit Issued for Subsidiaries 42
+--- [START OF PAGE 23] ---
+ii 
+ ARTICLE IVReserved 43
+ARTICLE VGENERAL LOAN PROVISIONS 43
+SECTION 5.1Interest 43
+SECTION 5.2Notice and Manner of Conversion or Continuation of Loans 44
+SECTION 5.3Fees 44
+SECTION 5.4Manner of Payment 45
+SECTION 5.5Evidence of Indebtedness 45
+SECTION 5.6Sharing of Payments by Lenders 46
+SECTION 5.7Administrative Agent’s Clawback 46
+SECTION 5.8Changed Circumstances 47
+SECTION 5.9Indemnity 50
+SECTION 5.10Increased Costs 50
+SECTION 5.11Taxes 51
+SECTION 5.12Mitigation Obligations; Replacement of Lenders 55
+SECTION 5.13Incremental Loans 56
+SECTION 5.14Cash Collateral 58
+SECTION 5.15Defaulting Lenders 58
+ARTICLE VICONDITIONS OF CLOSING AND BORROWING 60
+SECTION 6.1Conditions to Closing and Initial Extensions of Credit 60
+SECTION 6.2Conditions to All Extensions of Credit 64
+ARTICLE VIIREPRESENTATIONS AND WARRANTIES OF THE CREDIT PARTIES64
+SECTION 7.1Organization; Power; Qualification 64
+SECTION 7.2Ownership 65
+SECTION 7.3Authorization; Enforceability 65
+SECTION 7.4Compliance of Agreement, Loan Documents and Borrowing with
+Laws, Etc 65
+SECTION 7.5Compliance with Law; Governmental Approvals 65
+SECTION 7.6Tax Returns and Payments 66
+SECTION 7.7Intellectual Property Matters 66
+SECTION 7.8Environmental Matters 66
+SECTION 7.9Employee Benefit Matters 67
+SECTION 7.10Margin Stock 68
+SECTION 7.11Government Regulation 68
+SECTION 7.12Material Contracts 68
+SECTION 7.13Employee Relations 68
+--- [START OF PAGE 24] ---
+--- [START OF PAGE 25] ---
+iii 
+ SECTION 7.14Burdensome Provisions 69
+SECTION 7.15Financial Statements 69
+SECTION 7.16No Material Adverse Change 69
+SECTION 7.17Solvency 69
+SECTION 7.18Title to Properties 69
+SECTION 7.19Litigation 69
+SECTION 7.20Anti-Corruption Laws; Anti-Money Laundering Laws; Sanctions and
+Outbound Investment Rules 69
+SECTION 7.21Absence of Defaults 70
+SECTION 7.22ESOP 70
+SECTION 7.23Senior Indebtedness Status 71
+SECTION 7.24Disclosure 71
+ARTICLE VIIIAFFIRMATIVE COVENANTS 72
+SECTION 8.1Financial Statements and Budgets 72
+SECTION 8.2Certificates; Other Reports 73
+SECTION 8.3Notice of Litigation and Other Matters 73
+SECTION 8.4Preservation of Corporate Existence and Related Matters 75
+SECTION 8.5Maintenance of Property and Licenses 75
+SECTION 8.6Insurance 75
+SECTION 8.7Accounting Methods and Financial Records 76
+SECTION 8.8Payment of Taxes and Other Obligations 76
+SECTION 8.9Compliance with Laws and Approvals 76
+SECTION 8.10Environmental Laws 76
+SECTION 8.11Compliance with ERISA 76
+SECTION 8.12Compliance with Material Contracts 76
+SECTION 8.13Visits and Inspections 76
+SECTION 8.14Additional Subsidiaries 77
+SECTION 8.15Depository Bank 77
+SECTION 8.16Use of Proceeds 78
+SECTION 8.17ESOP 78
+SECTION 8.18Compliance with Anti-Corruption Laws; Beneficial Ownership
+Regulation, Anti-Money Laundering Laws and Sanctions 78
+SECTION 8.19Further Assurances 78
+SECTION 8.20Post-Closing Matters 79
+SECTION 8.21Lender Meetings 79
+--- [START OF PAGE 26] ---
+--- [START OF PAGE 27] ---
+iv 
+ ARTICLE IXNEGATIVE COVENANTS 79
+SECTION 9.1Indebtedness 79
+SECTION 9.2Liens 80
+SECTION 9.3Investments 81
+SECTION 9.4Fundamental Changes 82
+SECTION 9.5Asset Dispositions 83
+SECTION 9.6Restricted Payments 84
+SECTION 9.7Transactions with Affiliates 84
+SECTION 9.8Accounting Changes; Organizational Documents 84
+SECTION 9.9Payments and Modifications of Subordinated Indebtedness 85
+SECTION 9.10No Further Negative Pledges; Restrictive Agreements 85
+SECTION 9.11ESOP Matters 86
+SECTION 9.12Sale of Accounts 86
+SECTION 9.13Sale Leasebacks 86
+SECTION 9.14Capital Expenditures 86
+SECTION 9.15Financial Covenants 86
+SECTION 9.16No Amendment to ESOP Documentation 87
+SECTION 9.17Limitations Regarding Outbound Investment Rules 87
+ARTICLE XDEFAULT AND REMEDIES 87
+SECTION 10.1Events of Default 87
+SECTION 10.2Remedies 89
+SECTION 10.3Rights and Remedies Cumulative; Non-Waiver; etc 90
+SECTION 10.4Crediting of Payments and Proceeds 91
+SECTION 10.5Administrative Agent May File Proofs of Claim 91
+SECTION 10.6Credit Bidding 92
+ARTICLE XITHE ADMINISTRATIVE AGENT 92
+SECTION 11.1Appointment and Authority 92
+SECTION 11.2Rights as a Lender 93
+SECTION 11.3Exculpatory Provisions 93
+SECTION 11.4Reliance by the Administrative Agent 94
+SECTION 11.5Delegation of Duties 94
+SECTION 11.6Resignation of Administrative Agent 95
+SECTION 11.7Non-Reliance on Administrative Agent and Other Lenders 96
+SECTION 11.8No Other Duties, Etc 96
+SECTION 11.9Collateral and Guaranty Matters 96
+--- [START OF PAGE 28] ---
+--- [START OF PAGE 29] ---
+v 
+ SECTION 11.10Secured Hedge Agreements and Secured Cash Management
+Agreements 97
+SECTION 11.11[Reserved.] 97
+SECTION 11.12Erroneous Payments 97
+ARTICLE XIIMISCELLANEOUS 99
+SECTION 12.1Notices 99
+SECTION 12.2Amendments, Waivers and Consents 101
+SECTION 12.3Expenses; Indemnity 103
+SECTION 12.4Right of Setoff 105
+SECTION 12.5Governing Law; Jurisdiction, Etc 105
+SECTION 12.6Waiver of Jury Trial 106
+SECTION 12.7Reversal of Payments 106
+SECTION 12.8Injunctive Relief 107
+SECTION 12.9Successors and Assigns; Participations 107
+SECTION 12.10Treatment of Certain Information; Confidentiality 110
+SECTION 12.11Performance of Duties 111
+SECTION 12.12All Powers Coupled with Interest 111
+SECTION 12.13Survival 111
+SECTION 12.14Titles and Captions 112
+SECTION 12.15Severability of Provisions 112
+SECTION 12.16Counterparts; Integration; Effectiveness; Electronic Execution 112
+SECTION 12.17Term of Agreement 113
+SECTION 12.18USA PATRIOT Act; Anti-Money Laundering Laws 113
+SECTION 12.19Independent Effect of Covenants 113
+SECTION 12.20No Advisory or Fiduciary Responsibility 113
+SECTION 12.21Amendment and Restatement; No Novation 114
+SECTION 12.22Inconsistencies with Other Documents 115
+SECTION 12.23Acknowledgement and Consent to Bail-In of Affected Financial
+Institutions 115
+SECTION 12.24Certain ERISA Matters 115
+SECTION 12.25Acknowledgement Regarding Any Supported QFCs 116
+--- [START OF PAGE 30] ---
+viEXHIBITS
+Exhibit A-1 -Form of Revolving Credit Note
+Exhibit A-2 -Form of Swingline Note
+Exhibit B -Form of Notice of Borrowing
+Exhibit C -Form of Notice of Account Designation
+Exhibit D -Form of Notice of Prepayment
+Exhibit E -Form of Notice of Conversion/Continuation
+Exhibit F -Form of Officer’s Compliance Certificate
+Exhibit G -Form of Assignment and Assumption
+Exhibit H-1 -Form of U.S. Tax Compliance Certificate (Non-
+Partnership Foreign Lenders)
+Exhibit H-2 -Form of U.S. Tax Compliance Certificate (Non-
+Partnership Foreign Participants)
+Exhibit H-3 -Form of U.S. Tax Compliance Certificate (Foreign
+Participant Partnerships)
+Exhibit H-4 -Form of U.S. Tax Compliance Certificate (Foreign Lender
+Partnerships)
+Exhibit I -Form of Joinder Agreement
+SCHEDULES
+Schedule 1.1 -Commitments and Commitment Percentages
+Schedule 7.1 -Jurisdictions of Organization and Qualification
+Schedule 7.2 -Subsidiaries and Capitalization
+Schedule 7.6 -Tax Matters
+Schedule 7.9 -ERISA Plans
+Schedule 7.12 -Material Contracts
+Schedule 7.13 -Labor and Collective Bargaining Agreements
+Schedule 7.18 -Real Property
+Schedule 7.19 -Litigation
+Schedule 8.20 -Post-Closing Matters
+Schedule 9.1 -Existing Indebtedness
+Schedule 9.2 -Existing Liens
+Schedule 9.3 -Existing Loans, Advances and Investments
+Schedule 9.7 -Transactions with Affiliates
+Schedule 12.21 -Existing Letters of Credit
+--- [START OF PAGE 31] ---
+AMENDED AND RESTATED CREDIT AGREEMENT, dated as of June 28, 2023, by and
+among MAYVILLE ENGINEERING COMPANY, INC., a Wisconsin corporation (“Mayville” or the
+“Borrower”), the lenders who are party to this Agreement and the lenders who may become a party to
+this Agreement pursuant to the terms hereof, as Lenders, and WELLS FARGO BANK, NATIONAL
+ASSOCIATION, a national banking association, as Administrative Agent for the Lenders.
+STATEMENT OF PURPOSE
+The Borrower, the lenders party thereto, and WELLS FARGO BANK, NATIONAL
+ASSOCIATION, a national banking association, as administrative agent for such lenders, are party to
+that certain Amended and Restated Credit Agreement dated as of September 26, 2019 (as amended to
+date, the “Existing Credit Agreement”).  
+The Borrower has requested, and subject to the terms and conditions set forth in this
+Agreement, the Administrative Agent and the Lenders have agreed to extend certain credit facilities
+to the Borrower to be used, in part, to restructure, and to increase, the indebtedness and other
+obligations outstanding under the Existing Credit Agreement and amend and restate the Existing
+Credit Agreement in its entirety.
+NOW, THEREFORE, for good and valuable consideration, the receipt and sufficiency of
+which are hereby acknowledged by the parties hereto, such parties hereby agree as follows:
+ARTICLE I
+DEFINITIONS
+SECTION 1.1 Definitions.  The following terms when used in this Agreement shall
+have the meanings assigned to them below:
+“Accu-Fab Acquisition” means the contemplated Acquisition by the Borrower of all of the
+outstanding Equity Interests of Accu-Fab, LLC, a Delaware limited liability company, from Tide
+Rock Yieldco, LLC, a Delaware limited liability company, pursuant to that certain Purchase
+Agreement, dated as of May 23, 2025, by and among the Borrower, Accu-Fab, LLC and Tide Rock
+Yieldco, LLC.  
+“Acquisition” means any transaction, or any series of related transactions, consummated on
+or after the date of this Agreement, by which any Credit Party or any of its </t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>{
+  "errors": [
+    {
+      "location": "Page 33, Definitions - Section 1.1 Applicable Margin row",
+      "error": "Garbled/ambiguous line for Applicable Margin Level I; the text shows 'I Greater than or equal to 3.252.75%', which appears to merge/omit the ratio threshold and the first margin value.",
+      "suggestion": "Correct Level I row to 'I Greater than or equal to 3.25 to 1.00; SOFR margin 2.75%; Base Rate margin 1.75%; Commitment Fee 0.35%.'",
+      "exact_quote": "I Greater than or equal to 3.252.75% 1.75% 0.35%"
+    },
+    {
+      "location": "Page 85, Definitions - Term SOFR",
+      "error": "Definition of Term SOFR appears incomplete on this page; line reads '“Term SOFR” means,' with the actual definition continuing on a subsequent page.",
+      "suggestion": "Insert the complete Term SOFR definition on Page 85 or ensure the full definition is contiguous on a single page.",
+      "exact_quote": "“Term SOFR” means,"
+    },
+    {
+      "location": "Page 45, Definitions - Investment Company Act",
+      "error": "Statutory citation for Investment Company Act is incorrect; it currently cites '15 U.S.C. § 80(a) (1), et seq.' instead of the correct '15 U.S.C. § 80a-1 et seq.'",
+      "suggestion": "Correct the citation to '15 U.S.C. § 80a-1 et seq.'",
+      "exact_quote": "Investment Company Act” means the Investment Company Act of 1940 (15 U.S.C. § 80(a) (1), et seq.)."
+    },
+    {
+      "location": "Page 2, [START OF PAGE 2] - stray line",
+      "error": "Stray isolated character '1' appears on its own line, likely a formatting placeholder or stray artifact.",
+      "suggestion": "Remove the stray '1' line or replace with proper page formatting as intended.",
+      "exact_quote": "1"
+    },
+    {
+      "location": "Annex A (Pages 19-20)",
+      "error": "Annex A totals line shows 'Total $350,000,000.00100.000000000%', i.e., missing space between the currency amount and percentage and inconsistent formatting.",
+      "suggestion": "Insert a space to read 'Total $350,000,000.00 100.000000000%', ensuring consistent formatting with other lines.",
+      "exact_quote": "Total $350,000,000.00100.000000000%"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance backend logging for AI prompts, raw output, and locator results, and improve frontend log display.
</commit_message>
<xml_diff>
--- a/backend/audit_logs.xlsx
+++ b/backend/audit_logs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5813,6 +5813,1994 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-01-05 23:08:46</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>gpt-5.2-2025-12-11</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ce8d474d-b925-4719-af5f-6cea14551993.pdf</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document f...</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document fragment.
+Input: The attached text from a contract.
+CRITICAL INSTRUCTIONS:
+1. **Assume Isolation with Common Sense**: Do NOT assume missing definitions exist in other documents. However, IGNORE common commercial lending terms typically defined in a base Credit Agreement (e.g., "Borrower", "Administrative Agent", "Lender", "Business Day", "Dollars", "GAAP", "Material Adverse Effect"). Only flag specific, deal-specific, or unusual capitalized terms that are undefined.
+2. **Logic Check:** Check all math and logic tables.
+3. **Drafting Errors:** Find any placeholders like "[__]" or blank lines that were forgotten.
+4. **Exact Quotes:** For every error, you MUST provide the `exact_quote` from the text that contains the error. This is used for highlighting.
+Output Format:
+Return ONLY a valid JSON object with the following structure:
+{
+  "errors": [
+    {
+      "location": "Page 3, Section 2.1",
+      "error": "Description of the error",
+      "suggestion": "Suggested fix",
+      "exact_quote": "Exact text substring to highlight in red"
+    }
+  ]
+}
+If no errors are found, return {"errors": []}.
+--- CONTRACT TEXT BEGINS ---
+--- [START OF PAGE 1] ---
+EX-4.1 3 d45101 1dex41.htm EX-4.1
+Exhibit 4.1
+CAPITAL ONE PRIME AUTO RECEIVABLES TRUST 2023-1
+Class A-1 4.900% Auto Loan Asset Backed Notes
+Class A-2 5.20% Auto Loan Asset Backed Notes
+Class A-3 4.87% Auto Loan Asset Backed Notes
+Class A-4 4.76% Auto Loan Asset Backed Notes
+Class B 5.07% Auto Loan Asset Backed Notes
+Class C 5.36% Auto Loan Asset Backed Notes
+Class D 6.34% Auto Loan Asset Backed Notes
+INDENTURE
+Dated as of February 23, 2023
+WILMINGTON TRUST, NATIONAL ASSOCIATION,
+as the Indenture Trustee
+--- [START OF PAGE 2] ---
+CROSS REFERENCE TABLE1
+TIA
+Section     Indenture
+Section
+310   (a) (1)   6.11
+  (a) (2)   6.11
+  (a) (3)   6.10; 6.11
+  (a) (4)   N.A.2
+  (a) (5)   6.11
+  (b)   6.8; 6.11
+  (c)   N.A.
+311   (a)   6.12
+  (b)   6.12
+  (c)   N.A.
+312   (a)   7.1
+  (b)   7.2
+  (c)   7.2
+313   (a)   7.3
+  (b) (1)   7.3
+  (b) (2)   7.3
+  (c)   7.3
+  (d)   7.3
+314   (a)   3.9
+  (b)   11.1, 3.6
+  (c) (1)   11.1
+  (c) (2)   11.1
+  (c) (3)   11.1
+  (d)   11.1
+  (e)   11.1
+  (f)   N.A.
+315   (a)   6.1(b)
+  (b)   6.5
+  (c)   6.1(a)
+  (d)   6.1(c)
+  (e)   5.13
+316   (a) (1) (A)   5.11
+  (a) (1) (B)   5.12
+  (a) (2)   N.A.
+  (b)   5.7
+  (c)   5.6(b)
+317   (a) (1)   5.3(b)
+  (a) (2)   5.3(d)
+  (b)   3.3
+318   (a)   11.7 
+1 Note: This Cross Reference Table shall not, for any purpose, be deemed to be part of this Indenture.
+2 N.A. means Not Applicable.
+COPAR 2023-1 Indenture
+--- [START OF PAGE 3] ---
+TABLE OF CONTENTS
+     Page 
+ARTICLE I  DEFINITIONS AND INCORPORATION BY REFERENCE    2 
+Section 1.1 Definitions    2 
+Section 1.2 Incorporation by Reference of Trust Indenture Act    2 
+Section 1.3 Other Interpretive Provisions    2 
+ARTICLE II  THE NOTES    3 
+Section 2.1 Form    3 
+Section 2.2 Execution, Authentication and Delivery    3 
+Section 2.3 Temporary Notes    4 
+Section 2.4 Registration of Transfer and Exchange    4 
+Section 2.5 Mutilated, Destroyed, Lost or Stolen Notes    6 
+Section 2.6 Persons Deemed Owners    6 
+Section 2.7 Payment of Principal and Interest; Defaulted Interest    7 
+Section 2.8 Cancellation    7 
+Section 2.9 Release of Collateral    8 
+Section 2.10 Book-Entry Notes    8 
+Section 2.11 Notices to Clearing Agency    9 
+Section 2.12 Definitive Notes    9 
+Section 2.13 Authenticating Agents    10 
+Section 2.14 Paying Agent    10 
+Section 2.15 Tax and Accounting Treatment    11 
+Section 2.16 Certain Transfer Restrictions on all Classes of the Notes    11 
+Section 2.17 Certain Transfer Restrictions    12 
+Section 2.18 Transfer Restrictions on Certain Notes Upon a Sale of a Certificate    12 
+Section 2.19 Certain Transfer Restrictions on the 144A Notes    13 
+ARTICLE III  COVENANTS    17 
+Section 3.1 Payment of Principal and Interest    17 
+Section 3.2 Maintenance of Office or Agency    17 
+Section 3.3 Money for Payments to Be Held in Trust    17 
+Section 3.4 Existence    19 
+Section 3.5 Protection of Collateral    19 
+COPAR 2023-1 Indenture
+-i-
+--- [START OF PAGE 4] ---
+TABLE OF CONTENTS
+(continued)
+     Page 
+Section 3.6 Opinions as to Collateral    20 
+Section 3.7 Performance of Obligations; Servicing of Receivables    20 
+Section 3.8 Negative Covenants    21 
+Section 3.9 Annual Compliance Statement    22 
+Section 3.10 Restrictions on Certain Other Activities    23 
+Section 3.11 Restricted Payments    23 
+Section 3.12 Notice of Events of Default    23 
+Section 3.13 Further Instruments and Acts    23 
+Section 3.14 Compliance with Laws    23 
+Section 3.15 Removal of Administrator    23 
+Section 3.16 Perfection Representations, Warranties and Covenants    24 
+Section 3.17 Investment Company Act Representation    24 
+ARTICLE IV  SATISFACTION AND DISCHARGE    24 
+Section 4.1 Satisfaction and Discharge of Indenture    24 
+Section 4.2 Application of Trust Money    25 
+Section 4.3 Repayment of Monies Held by Paying Agent    25 
+ARTICLE V  REMEDIES    25 
+Section 5.1 Events of Default    25 
+Section 5.2 Acceleration of Maturity; Waiver of Event of Default    26 
+Section 5.3 Collection of Indebtedness and Suits for Enforcement by the Indenture Trustee    27 
+Section 5.4 Remedies; Priorities    29 
+Section 5.5 Optional Preservation of the Collateral    32 
+Section 5.6 Limitation of Suits    32 
+Section 5.7 Rights of Noteholders to Receive Principal and Interest    33 
+Section 5.8 Restoration of Rights and Remedies    33 
+Section 5.9 Rights and Remedies Cumulative    33 
+Section 5.10 Delay or Omission Not a Waiver    33 
+Section 5.11 Control by Noteholders    34 
+Section 5.12 Waiver of Past Defaults    34 
+Section 5.13 Undertaking for Costs    35 
+COPAR 2023-1 Indenture
+-ii-
+--- [START OF PAGE 5] ---
+TABLE OF CONTENTS
+(continued)
+     Page 
+Section 5.14 Waiver of Stay or Extension Laws    35 
+Section 5.15 Action on Notes    35 
+Section 5.16 Performance and Enforcement of Certain Obligations    35 
+Section 5.17 Sale of Collateral    36 
+ARTICLE VI  THE INDENTURE TRUSTEE    37 
+Section 6.1 Duties of the Indenture Trustee    37 
+Section 6.2 Rights of the Indenture Trustee    38 
+Section 6.3 Individual Rights of the Indenture Trustee    40 
+Section 6.4 The Indenture Trustee’s Disclaimer    40 
+Section 6.5 Notice of Defaults    40 
+Section 6.6 Reports by the Paying Agent    40 
+Section 6.7 Compensation and Indemnity    40 
+Section 6.8 Removal, Resignation and Replacement of the Indenture Trustee    41 
+Section 6.9 Successor Indenture Trustee by Merger    42 
+Section 6.10 Appointment of Co-Indenture Trustee or Separate Indenture Trustee    43 
+Section 6.11 Eligibility; Disqualification    44 
+Section 6.12 Preferential Collection of Claims Against the Issuer    44 
+Section 6.13 Representations and Warranties    44 
+ARTICLE VII  NOTEHOLDERS’ LISTS AND REPORTS    45 
+Section 7.1 The Issuer to Furnish the Indenture Trustee Names and Addresses of Noteholders    45 
+Section 7.2 Preservation of Information; Communications to Noteholders    45 
+Section 7.3 Reports by the Indenture Trustee    45 
+Section 7.4 Statements to Certificateholders and Noteholders    45 
+Section 7.5 Noteholder Demand for Repurchase, Dispute Resolution    47 
+Section 7.6 Investor Action to Initiate an Asset Review    48 
+ARTICLE VIII ACCOUNTS, DISBURSEMENTS AND RELEASES    49 
+Section 8.1 Collection of Money    49 
+Section 8.2 Trust Accounts    49 
+COPAR 2023-1 Indenture
+-iii-
+--- [START OF PAGE 6] ---
+TABLE OF CONTENTS
+(continued)
+     Page 
+Section 8.3 General Provisions Regarding Accounts    51 
+Section 8.4 Additional Withdrawals and Deposits    54 
+Section 8.5 Distributions    54 
+Section 8.6 Release of Collateral    56 
+Section 8.7 Opinion of Counsel    56 
+ARTICLE IX  SUPPLEMENTAL INDENTURES    57 
+Section 9.1 Supplemental Indentures Without Consent of Noteholders    57 
+Section 9.2 Supplemental Indentures with Consent of Noteholders    58 
+Section 9.3 Execution of Supplemental Indentures    59 
+Section 9.4 Effect of Supplemental Indenture    60 
+Section 9.5 Conformity with Trust Indenture Act    60 
+Section 9.6 Reference in Notes to Supplemental Indentures    60 
+ARTICLE X  REDEMPTION OF NOTES    60 
+Section 10.1 Redemption    60 
+Section 10.2 Form of Redemption Notice    61 
+Section 10.3 Notes Payable on Redemption Date    61 
+ARTICLE XI  MISCELLANEOUS    62 
+Section 11.1 Compliance Certificates and Opinions, etc.    62 
+Section 11.2 Form of Documents Delivered to the Indenture Trustee    63 
+Section 11.3 Acts of Noteholders    64 
+Section 11.4 Notices    65 
+Section 11.5 Notices to Noteholders; Waiver    65 
+Section 11.6 Alternate Payment and Notice Provisions    65 
+Section 11.7 Conflict with Trust Indenture Act    65 
+Section 11.8 Information Requests    66 
+Section 11.9 Effect of Headings and Table of Contents    66 
+Section 11.10 Successors and Assigns    66 
+Section 11.11 Separability    66 
+Section 11.12 Benefits of Indenture    66 
+Section 11.13 Legal Holidays    66 
+COPAR 2023-1 Indenture
+-iv-
+--- [START OF PAGE 7] ---
+TABLE OF CONTENTS
+(continued)
+     Page 
+Section 11.14 GOVERNING LAW    66 
+Section 11.15 Counterparts    66 
+Section 11.16 Recording of Indenture    67 
+Section 11.17 Trust Obligation    67 
+Section 11.18 No Petition    67 
+Section 11.19 Submission to Jurisdiction; Waiver of Jury Trial    68 
+Section 11.20 Subordination of Claims    68 
+Section 11.21 U.S.A Patriot Act    69 
+Section 11.22 Beneficial Ownership    69 
+Section 11.23 Limitation of Liability    69 
+ARTICLE XII  COMPLIANCE WITH THE FDIC RULE    70 
+Section 12.1 Purpose    70 
+Section 12.2 Requirements of the FDIC Rule    71 
+Section 12.3 Performance    72 
+Section 12.4 Actions Upon Repudiation    73 
+Section 12.5 Notice    75 
+Section 12.6 Reservation of Rights    75 
+Schedule I  Perfection Representations, Warranties and Covenants
+Exhibit A  Form of Notes
+COPAR 2023-1 Indenture
+-v-
+--- [START OF PAGE 8] ---
+This INDENTURE, dated as of February 23, 2023 (as amended, supplemented, or otherwise modified and in effect from time to time, this
+“Indenture”), is between CAPITAL ONE PRIME AUTO RECEIVABLES TRUST 2023-1, a Delaware statutory trust (the “Issuer”), and Wilmington
+Trust, National Association, a national banking association, solely as trustee and not in its individual capacity (the “Indenture Trustee”).
+Each party agrees as follows for the benefit of the other party and the equal and ratable benefit of the Holders of the Issuer’s Class A-1
+4.900% Auto Loan Asset Backed Notes (the “Class A-1 Notes”), Class A-2 5.20% Auto Loan Asset Backed Notes (the “Class A-2 Notes”), Class A-3
+4.87% Auto Loan Asset Backed Notes (the “Class A-3 Notes”), Class A-4 4.76% Auto Loan Asset Backed Notes (the “Class A-4 Notes”, and together
+with the Class A-1 Notes, the Class A-2 Notes and the Class A-3 Notes, the “Class A Notes”), Class B 5.07% Auto Loan Asset Backed Notes (the
+“Class B Notes”), Class C 5.36% Auto Loan Asset Backed Notes (the “Class C Notes”) and Class D 6.34% Auto Loan Asset Backed Notes (the
+“Class D Notes”, and together with the Class A-1 Notes, the Class A-2 Notes, the Class A-3 Notes, the Class A-4 Notes, the Class B Notes and the
+Class C Notes, the “Notes”).
+GRANTING CLAUSE
+The Issuer, to secure the payment of principal of and interest on, and any other amounts owing in respect of, the Notes equally and ratably
+without prejudice, priority or distinction except as set forth herein, and to secure compliance with the provisions of this Indenture, hereby Grants in trust
+to the Indenture Trustee on the Closing Date, as trustee for the benefit of the Noteholders, all of the Issuer’s right, title and interest, whether now owned
+or hereafter acquired, in and to (i) the Trust Estate and (ii) all present and future claims, demands, causes and choses in action in respect of any or all of
+the Trust Estate and all payments on or under and all proceeds of every kind and nature whatsoever in respect of any or all of the Trust Estate, including
+all proceeds of the conversion, voluntary or involuntary, into cash or other liquid property, all cash proceeds, accounts, accounts receivable, notes, drafts,
+acceptances, chattel paper, checks, deposit accounts, insurance proceeds, condemnation awards, rights to payment of any and every kind and other forms
+of obligations and receivables, instruments, securities, financial assets and other property which at any time constitute all or part of or are included in the
+proceeds of any of the Trust Estate (collectively, the “Collateral”).
+The Indenture Trustee, on behalf of the Noteholders, acknowledges the foregoing Grant, accepts the trusts under this Indenture and agrees
+to perform its duties required in this Indenture in accordance with the provisions of this Indenture.
+The foregoing Grant is made in trust to secure (i) the payment of principal of and interest on, and any other amounts owing in respect of,
+the Notes, equally and ratably without prejudice, priority or distinction except as set forth herein and (ii) compliance with the provisions of this
+Indenture, all as provided in this Indenture.
+Without limiting the foregoing Grant, any Receivable repurchased or purchased by (a) the Servicer pursuant to Section 3.6 of the Servicing
+Agreement or (b) by the Bank pursuant to Section 3.4 of the Purchase Agreement shall be deemed to be automatically released from the lien of this
+Indenture without any action being taken by the Indenture Trustee upon payment by the applicable purchaser of the related Repurchase Price for such
+Repurchased Receivable.
+COPAR 2023-1 Indenture
+--- [START OF PAGE 9] ---
+ARTICLE I
+DEFINITIONS AND INCORPORATION BY REFERENCE
+SECTION 1.1 Definitions. Capitalized terms are used in this Indenture as defined in Appendix A to the Sale Agreement, dated as of the
+date hereof (as amended, supplemented, or otherwise modified and in effect from time to time, the “Sale Agreement”), between the Issuer and Capital
+One Auto Receivables, LLC, which also contains rules as to usage that are applicable herein.
+SECTION 1.2 Incorporation by Reference of Trust Indenture Act. Whenever this Indenture refers to a provision of the TIA, the provision
+is incorporated by reference in and made a part of this Indenture. The following TIA terms used in this Indenture have the following meanings:
+“Commission” means the Securities and Exchange Commission.
+“indenture securities” means the Notes.
+“indenture security holder” means a Noteholder.
+“indenture to be qualified” means this Indenture.
+“indenture trustee” or “institutional trustee” means the Indenture Trustee.
+“obligor” on the indenture securities means the Issuer and any other obligor on the indenture securities.
+All other TIA terms used in this Indenture that are defined by the TIA, defined by TIA reference to another statute or defined by
+Commission rule have the meaning assigned to them by such definitions.
+SECTION 1.3 Other Interpretive Provisions. All terms defined in this Indenture shall have the defined meanings when used in any
+certificate or other document delivered pursuant hereto unless otherwise defined therein. For purposes of this Indenture and all such certificates and
+other documents, unless the context otherwise requires: (a) accounting terms not otherwise defined in this Indenture, and accounting terms partly
+defined in this Indenture to the extent not defined, shall have the respective meanings given to them under GAAP (provided, that, to the extent that the
+definitions in this Indenture and GAAP conflict, the definitions in this Indenture shall control); (b) terms defined in Article 9 of the UCC as in effect in
+the relevant jurisdiction and not otherwise defined in this Indenture are used as defined in that Article; (c) the words “hereof,” “herein” and “hereunder”
+and words of similar import refer to this Indenture as a whole and not to any particular provision of this Indenture; (d) references to any Article, Section,
+Schedule, Appendix or Exhibit are references to Articles, Sections, Schedules, Appendices and Exhibits in or to this Indenture and references to any
+paragraph, subsection, clause or other subdivision within any Section or definition refer to such paragraph, subsection, clause or other
+COPAR 2023-1 Indenture
+-2-
+--- [START OF PAGE 10] ---
+subdivision of such Section or definition; (e) the term “including” and all variations thereof means “including without limitation”; (f) except as
+otherwise expressly provided herein, references to any law or regulation refer to that law or regulation as amended from time to time and include any
+successor law or regulation; (g) references to any Person include that Person’s successors and assigns and (h) headings are for purposes of reference
+only and shall not otherwise affect the meaning or interpretation of any provision hereof.
+ARTICLE II
+THE NOTES
+SECTION 2.1 Form. The Class A-1 Notes, Class A-2 Notes, Class A-3 Notes, Class A-4 Notes, Class B Notes, Class C Notes and Class D
+Notes, in each case together with the Indenture Trustee’s certificate of authentication, shall be in substantially the form set forth in Exhibit A hereto, with
+such appropriate insertions, omissions, substitutions and other variations as are required or permitted by this Indenture and may have such letters,
+numbers or other marks of identification and such legends or endorsements placed thereon as may, consistently herewith, be determined by the officers
+executing the Notes, as evidenced by their execution of the Notes. Any portion of the text of any Note may be set forth on the reverse thereof, with an
+appropriate reference thereto on the face of the Note.
+Each Note shall be dated the date of its authentication. The terms of the Notes set forth in Exhibit A hereto are part of the terms of this
+Indenture.
+SECTION 2.2 Execution, Authentication and Delivery. The Notes shall be executed on behalf of the Issuer by any of its Authorized
+Officers.
+Notes bearing the signature of individuals who were at any time Authorized Officers of the Issuer shall bind the Issuer, notwithstanding
+that such individuals or any of them have ceased to hold such offices prior to the authentication and delivery of such Notes or did not hold such offices
+at the date of such Notes.
+The Indenture Trustee shall, upon Issuer Order, authenticate and deliver Class A-1 Notes for original issue in an Initial Note Balance of
+$234,000,000, Class A-2 Notes for original issue in an Initial Note Balance of $508,100,000, Class A-3 Notes for original issue in an Initial Note
+Balance of $475,000,000, Class A-4 Notes for original issue in an Initial Note Balance of $98,700,000, Class B Notes for original issue in an Initial Note
+Balance of $13,560,000, Class C Notes for original issue in an Initial Note Balance of $13,560,000 and Class D Notes for original issue in an Initial
+Note Balance of $13,560,000. The Note Balance of Class A-1 Notes, Class A-2 Notes, Class A-3 Notes, Class A-4 Notes, Class B Notes, Class C Notes
+and Class D Notes Outstanding at any time may not exceed such amounts except as provided in Section 2.5.
+Each Note shall be dated the date of its authentication. The Notes shall be issuable as registered Notes in the minimum denomination of
+$1,000 and in integral multiples of $1,000 in excess thereof (except for one Note of each Class which may be issued in a denomination other than an
+integral multiple of $1,000).
+COPAR 2023-1 Indenture
+-3-
+--- [START OF PAGE 11] ---
+No Note shall be entitled to any benefit under this Indenture or be valid or obligatory for any purpose, unless there appears on such Note a
+certificate of authentication substantially in the form provided for herein executed by the Indenture Trustee by the manual signature of one of its
+authorized signatories, and such certificate upon any Note shall be conclusive evidence, and the only evidence, that such Note has been duly
+authenticated and delivered hereunder.
+SECTION 2.3 Temporary Notes. Pending the preparation of Definitive Notes, the Issuer may execute, and upon receipt of an Issuer Order,
+the Indenture Trustee shall authenticate and deliver, temporary Notes which are printed, lithographed, typewritten, mimeographed or otherwise
+produced, of the tenor of the Definitive Notes in lieu of which they are issued and with such variations not inconsistent with the terms of this Indenture
+as the officers executing such Notes may determine, as evidenced by their execution of such Notes.
+If temporary Notes are issued, the Issuer shall cause Definitive Notes to be prepared without unreasonable delay. After the preparation of
+Definitive Notes, the temporary Notes shall be exchangeable for Definitive Notes upon surrender of the temporary Notes at the office or agency of the
+Issuer to be maintained as provided in Section 3.2, without charge to the Holder. Upon surrender for cancellation of any one or more temporary Notes,
+the Issuer shall execute and the Indenture Trustee upon Issuer Order shall authenticate and deliver in exchange therefor a like principal amount of
+Definitive Notes of authorized denominations. Until so exchanged, the temporary Notes shall in all respects be entitled to the same benefits under this
+Indenture as Definitive Notes.
+SECTION 2.4 Registration of Transfer and Exchange.
+(a) The Issuer shall cause to be kept a register (the “Note Register”) in which, subject to such reasonable regulations as it may prescribe,
+the Issuer shall provide for the registration of Notes and the registration of transfers of Notes. The Indenture Trustee shall initially be the “Note
+Registrar” for the purpose of registering Notes and transfers of Notes as herein provided. Upon any resignation of any Note Registrar, the Issuer shall
+promptly appoint a successor or, if it elects not to make such an appointment, assume the duties of Note Registrar.
+If a Person other than the Indenture Trustee is appointed by the Issuer as Note Registrar, the Issuer shall give the Indenture Trustee prompt written
+notice of the appointment of such Note Registrar and of the location, and any change in the location, of the Note Register, and the Indenture Trustee
+shall have the right to inspect the Note Register at all reasonable times and to obtain copies thereof, and the Indenture Trustee shall have the right to
+conclusively rely upon a certificate executed on behalf of the Note Registrar by a Responsible Officer thereof as to the names and addresses of the
+Noteholders and the principal amounts and number of such Notes.
+Notwithstanding the foregoing, for so long as Wilmington Trust, National Association is acting as the Indenture Trustee hereunder, it shall also act
+as the Note Registrar.
+(b) Upon surrender for registration of transfer of any Note at the office or agency of the Issuer to be maintained as provided in Section 3.2,
+if the requirements of Section 8-401 of the UCC are met, the Issuer shall execute and upon its written request the Indenture Trustee shall authenticate
+and the Noteholder shall obtain from the Indenture Trustee, in the name of the designated transferee or transferees, one or more new Notes, in any
+authorized denominations, of the same Class and a like Outstanding Note Balance.
+COPAR 2023-1 Indenture
+-4-
+--- [START OF PAGE 12] ---
+At the option of the related Noteholder, Notes may be exchanged for other Notes in any authorized denominations, of the same Class and a
+like Outstanding Note Balance, upon surrender of the Notes to be exchanged at such office or agency. Whenever any Notes are so surrendered for
+exchange, if the requirements of Section 8-401 of the UCC are met the Issuer shall execute and, upon Issuer Request, the Indenture Trustee shall
+authenticate and the related Noteholder shall obtain from the Indenture Trustee, the Notes which the Noteholder making the exchange is entitled to
+receive.
+(c) All Notes issued upon any registration of transfer or exchange of Notes shall be the valid obligations of the Issuer, evidencing the same
+debt, and entitled to the same benefits under this Indenture, as the Notes surrendered upon such registration of transfer or exchange.
+(d) Every Note presented or surrendered for registration of transfer or exchange shall be (i) duly endorsed by, or be accompanied by, a
+written instrument of transfer in form and substance satisfactory to the Issuer and the Indenture Trustee duly executed by the Noteholder thereof or its
+attorney-in-fact duly authorized in writing, with such signature guaranteed by an “eligible grantor institution” meeting the requirements of the Note
+Registrar which requirements include membership or participation in the Securities Transfer Agents Medallion Program (“STAMP”) or such other
+“signature guarantee program” as may be determined by the Note Registrar in addition to, or in substitution for, STAMP, all in accordance with the
+Exchange Act and (ii) accompanied by such other documents as the Indenture Trustee may require, including but not limited to the applicable IRS Form
+W-8 or W-9.
+(e) No service charge shall be made to a Noteholder for any registration of transfer or exchange of Notes, but the Issuer may require
+payment of a sum sufficient to cover any tax or other governmental charge that may be imposed in connection with any registration of transfer or
+exchange of Notes, other than exchanges pursuant to Section 2.3 or Section 9.6 not involving any transfer.
+(f) The Indenture Trustee shall have no obligation or duty to monitor, determine or inquire as to compliance with any restrictions on
+transfer imposed under this Indenture or under applicable law with respect to any transfer of any interest in any Note other than to require delivery of
+such certificates and other documentation or evidence as are expressly required by, and to do so if and when expressly required by, the terms of this
+Indenture, and to examine the same to determine substantial compliance as to form with the express requirements hereof.
+(g) The preceding provisions of this Section 2.4 notwithstanding, the Issuer shall not be required to make and the Note Registrar need not
+register transfers or exchanges of any Notes selected for redemption or of any Note for a period of fifteen (15) days preceding the Redemption Date or
+any Payment Date, as applicable.
+COPAR 2023-1 Indenture
+-5-
+--- [START OF PAGE 13] ---
+SECTION 2.5 Mutilated, Destroyed, Lost or Stolen Notes. If (i) any mutilated Note is surrendered to the Indenture Trustee, or the
+Indenture Trustee receives evidence to its satisfaction of the destruction, loss or theft of any Note, and (ii) there is delivered to the Indenture Trustee
+such security or indemnity as may be required by it to hold the Issuer and the Indenture Trustee harmless, then, in the absence of notice to the Issuer, the
+Note Registrar or the Indenture Trustee that such Note has been acquired by a “protected purchaser” (as contemplated by Article 8 of the UCC), and
+provided that the requirements of Section 8-405 of the UCC are met, the Issuer shall execute and upon its written request the Indenture Trustee shall
+authenticate and deliver, in exchange for or in lieu of any such mutilated, destroyed, lost or stolen Note, a replacement Note; provided that if any such
+destroyed, lost or stolen Note, but not a mutilated Note, shall have become or within seven (7) days shall be due and payable, or shall have been called
+for redemption, instead of issuing a replacement Note, the Issuer may upon delivery of the security or indemnity herein required pay such destroyed, lost
+or stolen Note when so due or payable or upon the Redemption Date without surrender thereof. If, after the delivery of such replacement Note or
+payment of a destroyed, lost or stolen Note pursuant to the proviso to the preceding sentence, a “protected purchaser” (as contemplated by Article 8 of
+the UCC) of the original Note in lieu of which such replacement Note was issued presents for payment such original Note, the Issuer and the Indenture
+Trustee shall be entitled to recover such replacement Note (or such payment) from the Person to whom it was delivered or any Person taking such
+replacement Note from such Person to whom such replacement Note was delivered or any assignee of such Person, except a “protected purchaser” (as
+contemplated by Article 8 of the UCC), and shall be entitled to recover upon the security or indemnity provided therefor to the extent of any loss,
+damage, cost or expense incurred by the Issuer or the Indenture Trustee in connection therewith.
+Upon the issuance of any replacement Note under this Section 2.5, the Issuer or the Indenture Trustee may require the payment by the
+Noteholder of a sum sufficient to cover any tax or other governmental charge that may be imposed in relation thereto and any other reasonable expenses
+(including the fees and expenses of the Indenture Trustee or the Note Registrar) connected therewith.
+Every replacement Note issued pursuant to this Section 2.5 in replacement of any mutilated, destroyed, lost or stolen Note shall constitute
+an original additional contractual obligation of the Issuer and shall be entitled to all the benefits of this Indenture equally and proportionately with any
+and all other Notes duly issued hereunder.
+The provisions of this Section 2.5 are exclusive and shall preclude (to the extent lawful) all other rights and remedies with respect to the
+replacement or payment of mutilated, destroyed, lost or stolen Notes.
+SECTION 2.6 Persons Deemed Owners. Prior to due presentment for registration of transfer of any Note, the Issuer, the Indenture Trustee
+and any agent of the Issuer or the Indenture Trustee shall treat the Person in whose name any Note is registered (as of the day of determination) as the
+owner of such Note for the purpose of receiving payments of principal of and interest, if any, on such Note and for all other purposes whatsoever,
+whether or not such Note be overdue, and neither the Issuer, the Indenture Trustee nor any agent of the Issuer or the Indenture Trustee shall be affected
+by notice to the contrary.
+COPAR 2023-1 Indenture
+-6-
+--- [START OF PAGE 14] ---
+SECTION 2.7 Payment of Principal and Interest; Defaulted Interest.
+(a) Each of the Notes shall accrue interest at its respective Interest Rate, and such interest shall be payable on each Payment Date as
+specified therein, subject to Sections 3.1 and 8.2. Any installment of interest or principal, if any, payable on any Note which is punctually paid or duly
+provided for by the Issuer on the applicable Payment Date shall be paid to the Person in whose name such Note (or one or more Predecessor Notes) is
+registered on the Record Date, by wire transfer in immediately available funds to the account designated in writing to the Indenture Trustee by such
+Person (or, if no such account is designated in writing to the Indenture Trustee by such Person, then by check mailed first-class, postage prepaid, to such
+Person’s address as it appears on the Note Register on such Record Date), except that, unless Definitive Notes have been issued pursuant to
+Section 2.12, with respect to Notes registered on the Record Date in the name of the nominee of the Clearing Agency (initially, such nominee to be
+Cede &amp; Co.), payment will be made by wire transfer in immediately available funds to the account designated by such nominee and except for the final
+installment of principal payable with respect to such Note on a Payment Date or on the Final Scheduled Payment Date for such Class (and except for the
+Redemption Price for any Note called for redemption pursuant to Section 10.1) which shall be payable as provided below. The funds represented by any
+such checks returned undelivered shall be held in accordance with Section 3.3.
+(b) The principal of each Note shall be payable in installments on each Payment Date as provided in Section 8.2. Notwithstanding the
+foregoing, the entire unpaid Note Balance and all accrued interest thereon shall be due and payable, if not previously paid, on the earlier of (i) the date
+on which an Event of Default shall have occurred and be continuing, if the Indenture Trustee or the Holders of a majority of the Outstanding Note
+Balance of the Controlling Class have declared the Notes to be immediately due and payable in the manner provided in Section 5.2 and (ii) with respect
+to any Class of Notes, on the Final Scheduled Payment Date for that Class. All principal payments on each Class of Notes shall be made pro rata to the
+Noteholders of such Class entitled thereto. The Indenture Trustee shall notify the Person in whose name a Note is registered at the close of</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>{
+  "errors": [
+    {
+      "location": "Page 2, header",
+      "error": "Footnote indicator appears to be concatenated to the title (missing space), creating a formatting/typographical error.",
+      "suggestion": "Insert a space before the footnote indicator (e.g., \"CROSS REFERENCE TABLE 1\").",
+      "exact_quote": "CROSS REFERENCE TABLE1"
+    },
+    {
+      "location": "Page 46, Section 6.2(f)",
+      "error": "Internal cross-reference appears incorrect: it references \"Section 3.12 of the Sale Agreement\" as covering Noteholders’/Note Owners’ right to communicate with each other, but the communication right is typically governed by TIA Section 312 and is addressed here in Section 7.2(b). This looks like a mistaken section number/citation.",
+      "suggestion": "Confirm the correct Sale Agreement section (if any) intended to be referenced, or replace with the correct Indenture section (e.g., Section 7.2(b)) or the correct statutory reference.",
+      "exact_quote": "pursuant to this Indenture (other than requests, demands or directions relating to an Asset Review as described in Section 7.6 hereof or to the Noteholders’ or Note Owners’ right to communication with each other as described in Section 3.12 of the Sale Agreement)"
+    },
+    {
+      "location": "Page 81, Section 12.4(e)(ii)",
+      "error": "Numbering error creates logical ambiguity: clause (ii) contains nested items labeled \"(i)\" and \"(ii)\" again (duplicate numbering within the same level).",
+      "suggestion": "Renumber the subclauses within Section 12.4(e)(ii) (e.g., change to (A) and (B), or (1) and (2)).",
+      "exact_quote": "(ii) the Computation Agent shall promptly, and no later than one Business Day after such damages have been paid by the FDIC,\n(i) compute the amount, if any, required to be withdrawn from available funds in the Reserve Account and transferred to the Principal Distribution\nAccount so that the amount on deposit in the Principal Distribution\nAccount shall equal the aggregate amount to be distributed as specified in\nSection 12.4(c), and (ii) promptly inform the Servicer, the Owner Trustee and\nthe Indenture Trustee (if a separate Person) in writing of such\ncomputations;"
+    },
+    {
+      "location": "Page 83, signature blocks",
+      "error": "Incomplete execution blocks: blank signature lines (\"By:\") and missing name/title fields suggest placeholders were not completed.",
+      "suggestion": "Complete the signature blocks with signatures, printed names, and titles (or remove if this is an exhibit/sample form).",
+      "exact_quote": "By:  \nName:\nTitle:"
+    },
+    {
+      "location": "Page 83, signature blocks (Issuer)",
+      "error": "Incomplete execution block for the Issuer (Owner Trustee signature line and name/title blank).",
+      "suggestion": "Complete the Issuer execution block with signature, printed name, and title.",
+      "exact_quote": "By:  \nName:\nTitle:"
+    },
+    {
+      "location": "Page 86, Exhibit A heading",
+      "error": "Bracketed placeholders remain in the form heading and indicate the form was not finalized for a specific Class of Notes.",
+      "suggestion": "Replace bracketed placeholders with the applicable class (or provide separate finalized forms for each Class).",
+      "exact_quote": "FORM OF CLASS [A-1] [A-2] [A-3] [A-4] [B] [C] [D] NOTES"
+    },
+    {
+      "location": "Page 86, Exhibit A - face of note",
+      "error": "Unfilled amount placeholder for principal/denomination on the face of the Note.",
+      "suggestion": "Insert the applicable registered principal amount.",
+      "exact_quote": "$___________________1"
+    },
+    {
+      "location": "Page 86, Exhibit A - face of note",
+      "error": "Unfilled note number placeholder.",
+      "suggestion": "Insert the note number.",
+      "exact_quote": "No. R-________"
+    },
+    {
+      "location": "Page 86, Exhibit A - face of note",
+      "error": "Unfilled CUSIP placeholder.",
+      "suggestion": "Insert the applicable CUSIP number (or remove if not applicable).",
+      "exact_quote": "CUSIP NO. ______________"
+    },
+    {
+      "location": "Page 86, Exhibit A - face of note",
+      "error": "Unfilled ISIN placeholder and formatting error (\"ISIN.\" instead of \"ISIN\").",
+      "suggestion": "Insert the applicable ISIN (or remove if not applicable) and correct punctuation to \"ISIN\".",
+      "exact_quote": "ISIN. ______________"
+    },
+    {
+      "location": "Page 88, Exhibit A - promise to pay",
+      "error": "Unfilled registered holder placeholder.",
+      "suggestion": "Insert the name of the registered holder (or use \"Cede &amp; Co.\" for global notes).",
+      "exact_quote": "pay to [______], or registered assigns"
+    },
+    {
+      "location": "Page 88, Exhibit A - promise to pay",
+      "error": "Unfilled principal sum placeholders.",
+      "suggestion": "Insert the principal sum in words and figures.",
+      "exact_quote": "the principal sum of [___] DOLLARS ($[___])"
+    },
+    {
+      "location": "Page 88, Exhibit A - Final Scheduled Payment Date",
+      "error": "Unfilled Final Scheduled Payment Date placeholder.",
+      "suggestion": "Insert the applicable Final Scheduled Payment Date for the relevant Class (or cross-reference the defined term if defined elsewhere).",
+      "exact_quote": "on the earliest of (i) [___] (the “Final Scheduled Payment Date”)"
+    },
+    {
+      "location": "Page 88, Exhibit A - interest accrual conventions",
+      "error": "Bracketed alternative interest accrual language remains (not finalized for the applicable class).",
+      "suggestion": "Select and retain the correct accrual convention for the applicable Class and delete the inapplicable bracketed text/footnote markers.",
+      "exact_quote": "Interest on this Note will accrue for each Payment Date from and including the [preceding Payment Date (or, in the case of\nthe initial Payment Date, from and including the Closing Date) to but excluding such Payment Date]2 [15th day of the prior calendar month (or, in the\ncase of the initial Payment Date from and including the Closing Date) to but excluding the 15th day of the calendar month in which such Payment Date\noccurs]3."
+    },
+    {
+      "location": "Page 89, Exhibit A - Note signature block",
+      "error": "Incomplete signature block for the Note form (missing date, signature, name, and title).",
+      "suggestion": "Complete the Note execution block or label as a specimen form if not intended to be executed.",
+      "exact_quote": "Dated:\n \nCAPITAL ONE PRIME AUTO RECEIVABLES TRUST\n2023-1\nBy: BNY MELLON TRUST OF DELAWARE, not in its\nindividual capacity but solely as Owner Trustee\nBy:  \nName:  \nTitle:"
+    },
+    {
+      "location": "Page 90, Exhibit A - certificate of authentication",
+      "error": "Incomplete authentication certificate (missing date and authorized signatory name/signature line completion).",
+      "suggestion": "Complete the authentication certificate fields for executed notes, or label as specimen form.",
+      "exact_quote": "Dated:\n \nWILMINGTON TRUST, NATIONAL ASSOCIATION,\na national banking association, not in its individual capacity\nbut solely as Indenture Trustee\nBy:  \n Authorized Signatory"
+    },
+    {
+      "location": "Page 91, Exhibit A - reverse of note",
+      "error": "Duplicate sentence appears twice consecutively (likely a drafting duplication).",
+      "suggestion": "Delete one of the duplicate sentences.",
+      "exact_quote": "All covenants and agreements\nmade by the Issuer in the Indenture are for the benefit of the Holders of the Class A Notes, Class B Notes, Class C Notes and the Class D Notes. All\ncovenants and agreements\nmade by the Issuer in the Indenture are for the benefit of the Holders of the Class A Notes, Class B Notes, Class C Notes and the Class D Notes."
+    },
+    {
+      "location": "Page 91, Exhibit A - reverse of note",
+      "error": "Unfilled Final Scheduled Payment Date placeholder repeated on the reverse of the Note.",
+      "suggestion": "Insert the applicable Final Scheduled Payment Date for the relevant Class (or cross-reference a defined term).",
+      "exact_quote": "on the earliest of (i) [___] (the “Final\nScheduled Payment Date”)"
+    },
+    {
+      "location": "Page 94, Exhibit A - assignment form",
+      "error": "Unfilled placeholder for attorney-in-fact name in assignment block.",
+      "suggestion": "Insert the attorney-in-fact name or replace with a standard form (e.g., \"the Note Registrar\").",
+      "exact_quote": "hereby irrevocably constitutes and appoints ______________________, attorney, to transfer said Note"
+    },
+    {
+      "location": "Page 94, Exhibit A - assignment form",
+      "error": "Blank date line in assignment block appears as an uncompleted placeholder.",
+      "suggestion": "Provide a completed date for executed assignments or format as a blank line without underscore placeholders if intended as a form.",
+      "exact_quote": "Dated: _____________"
+    },
+    {
+      "location": "Page 15, Section 2.9 (and elsewhere)",
+      "error": "Potential undefined deal-specific term: \"Independent Certificates\" is used as a defined concept, but no definition appears in this fragment (and it is not a common commercial lending base-credit-agreement term).",
+      "suggestion": "Add a definition of \"Independent Certificates\" in the applicable definitions section or replace with the intended defined term/reference.",
+      "exact_quote": "Independent Certificates in accordance with TIA Sections 314(c) and 314(d)(1)"
+    },
+    {
+      "location": "Page 53, Section 7.4",
+      "error": "Potential undefined deal-specific term: \"Relevant Trustee\" is used repeatedly, but no definition appears in this fragment (and it is not a standard base credit agreement term).",
+      "suggestion": "Define \"Relevant Trustee\" (and clarify which trustee acts when) or replace with the specific trustee name in each instance.",
+      "exact_quote": "On each Payment Date, the Relevant Trustee shall make the Servicer’s\nReport"
+    },
+    {
+      "location": "Page 12, Section 2.4(d) (and Page 94 assignment legend)",
+      "error": "Inconsistent terminology: the assignment legend uses \"eligible guarantor institution\" while Section 2.4(d) uses \"eligible grantor institution\". This inconsistency may create ambiguity as to the intended standard for signature guarantees.",
+      "suggestion": "Confirm the correct term and use it consistently (commonly \"eligible guarantor institution\").",
+      "exact_quote": "with such signature guaranteed by an “eligible grantor institution”"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-03 21:25:44</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ce7d57f0-362a-400c-b784-2c5ea3d4ca02.pdf</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document f...</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document fragment.
+Input: The attached text from a contract.
+CRITICAL INSTRUCTIONS:
+1. **Assume Isolation with Common Sense**: Do NOT assume missing definitions exist in other documents. However, IGNORE common commercial lending terms typically defined in a base Credit Agreement (e.g., "Borrower", "Administrative Agent", "Lender", "Business Day", "Dollars", "GAAP", "Material Adverse Effect"). Only flag specific, deal-specific, or unusual capitalized terms that are undefined.
+2. **Logic Check:** Check all math and logic tables.
+3. **Drafting Errors:** Find any placeholders like "[__]" or blank lines that were forgotten.
+4. **Exact Quotes:** For every error, you MUST provide the `exact_quote` from the text that contains the error. This is used for highlighting.
+Output Format:
+Return ONLY a valid JSON object with the following structure:
+{
+  "errors": [
+    {
+      "location": "Page 3, Section 2.1",
+      "error": "Description of the error",
+      "suggestion": "Suggested fix",
+      "exact_quote": "Exact text substring to highlight in red"
+    }
+  ]
+}
+If no errors are found, return {"errors": []}.
+--- CONTRACT TEXT BEGINS ---
+--- [START OF PAGE 1] ---
+FIRST AMENDMENT TO AMENDED AND RESTATED
+CREDIT AGREEMENT
+This document is a generated test file containing intentional legal drafting errors for AI training
+purposes.
+ARTICLE I: DEFINITIONS
+...
+"Applicable Margin" means the corresponding percentages per annum as set forth below based on
+the Consolidated Total Leverage Ratio:
+Pricing Level
+Consolidated Total Leverage Ratio
+SOFR Margin
+I
+Greater than or equal to 3.25 to 1.00
+2.75%
+II
+Greater than or equal to 2.60 to 1.00 but less than 3.25 to 1.00
+2.50%
+III
+Greater than or equal to 1.75 to 1.00 but less than 2.50 to 1.00
+2.25%
+IV
+Greater than or equal to 1.50 to 1.00 but less than 1.75 to 1.00
+2.00%
+V
+Less than 1.50 to 1.00
+1.75%
+"Cash Collateral" shall have a meaning correlative to the foregoing and shall include the proceeds of
+such cash collateral...
+(Note: "Cash Collateralize" is defined, but "Cash Collateralization" is NOT defined
+in this section.)
+SECTION 2.5 Permanent Reduction of the Revolving Credit
+Commitment
+The Borrower shall have the right at any time to terminate the Revolving Credit Commitment...
+Any reduction of the Revolving Credit Commitment to zero shall be accompanied by payment of all
+outstanding Revolving Credit Loans and furnishing of Cash Collateralization satisfactory to the
+Administrative Agent.
+SECTION 5.13 Incremental Loans
+At any time after the First Amendment Effective Date, the Borrower may by written notice to the
+Administrative Agent elect to request the establishment of one or more increases in the Revolving
+--- [START OF PAGE 2] ---
+Credit Commitments...
+Such notice shall be delivered to the Administrative Agent at its office in [__] (or such other location as
+the Administrative Agent may designate).
+The terms of such Incremental Revolving Credit Increase shall be subject to the documentation
+requirements set forth in Section 5.19.
+[End of Document]
+--- CONTRACT TEXT ENDS ---</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>{
+  "errors": [
+    {
+      "location": "Page 1, ARTICLE I: DEFINITIONS, 'Applicable Margin'",
+      "error": "There is a logical gap in the 'Applicable Margin' pricing table. A Consolidated Total Leverage Ratio between 2.50 to 1.00 and 2.60 to 1.00 (exclusive) is not covered by any pricing level, making the pricing indeterminate for ratios in that range.",
+      "suggestion": "Adjust the pricing levels to ensure all possible Consolidated Total Leverage Ratios are covered. For instance, modify 'III' to 'Greater than or equal to 1.75 to 1.00 but less than 2.60 to 1.00' or modify 'II' to 'Greater than or equal to 2.50 to 1.00 but less than 3.25 to 1.00'.",
+      "exact_quote": "Consolidated Total Leverage Ratio\nSOFR Margin\nI\nGreater than or equal to 3.25 to 1.00\n2.75%\nII\nGreater than or equal to 2.60 to 1.00 but less than 3.25 to 1.00\n2.50%\nIII\nGreater than or equal to 1.75 to 1.00 but less than 2.50 to 1.00\n2.25%"
+    },
+    {
+      "location": "Page 1, SECTION 2.5",
+      "error": "The capitalized term 'Cash Collateralization' is used but not defined in this document fragment, as explicitly noted by the document's own comment.",
+      "suggestion": "Define 'Cash Collateralization' in 'ARTICLE I: DEFINITIONS', or ensure it is clearly understood as a derivative of a defined term like 'Cash Collateral' or 'Cash Collateralize' if that is the intent.",
+      "exact_quote": "furnishing of Cash Collateralization satisfactory to the Administrative Agent."
+    },
+    {
+      "location": "Page 1, SECTION 5.13",
+      "error": "The capitalized term 'First Amendment Effective Date' is used but not defined in this document fragment.",
+      "suggestion": "Define 'First Amendment Effective Date' in 'ARTICLE I: DEFINITIONS'.",
+      "exact_quote": "At any time after the First Amendment Effective Date, the Borrower may by written notice to the"
+    },
+    {
+      "location": "Page 2, SECTION 5.13",
+      "error": "A placeholder '[__]' indicates missing information that needs to be filled in.",
+      "suggestion": "Specify the exact office location of the Administrative Agent.",
+      "exact_quote": "Such notice shall be delivered to the Administrative Agent at its office in [__] (or such other location as"
+    },
+    {
+      "location": "Page 2, SECTION 5.13",
+      "error": "The capitalized term 'Incremental Revolving Credit Increase' is used but not defined in this document fragment.",
+      "suggestion": "Define 'Incremental Revolving Credit Increase' in 'ARTICLE I: DEFINITIONS'.",
+      "exact_quote": "The terms of such Incremental Revolving Credit Increase shall be subject to the documentation"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-03 21:27:06</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>gpt-5.2-2025-12-11</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>c36be49b-2094-480f-86be-34b1112f0bc8.pdf</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document f...</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document fragment.
+Input: The attached text from a contract.
+CRITICAL INSTRUCTIONS:
+1. **Assume Isolation with Common Sense**: Do NOT assume missing definitions exist in other documents. However, IGNORE common commercial lending terms typically defined in a base Credit Agreement (e.g., "Borrower", "Administrative Agent", "Lender", "Business Day", "Dollars", "GAAP", "Material Adverse Effect"). Only flag specific, deal-specific, or unusual capitalized terms that are undefined.
+2. **Logic Check:** Check all math and logic tables.
+3. **Drafting Errors:** Find any placeholders like "[__]" or blank lines that were forgotten.
+4. **Exact Quotes:** For every error, you MUST provide the `exact_quote` from the text that contains the error. This is used for highlighting.
+Output Format:
+Return ONLY a valid JSON object with the following structure:
+{
+  "errors": [
+    {
+      "location": "Page 3, Section 2.1",
+      "error": "Description of the error",
+      "suggestion": "Suggested fix",
+      "exact_quote": "Exact text substring to highlight in red"
+    }
+  ]
+}
+If no errors are found, return {"errors": []}.
+--- CONTRACT TEXT BEGINS ---
+--- [START OF PAGE 1] ---
+EX-10.1 4 d45101 1dex101.htm EX-10.1
+Exhibit 10.1
+PURCHASE AGREEMENT
+dated as of February 23, 2023
+between
+CAPITAL ONE, NATIONAL ASSOCIATION
+and
+CAPITAL ONE AUTO RECEIVABLES, LLC,
+as Purchaser
+COPAR 2023-1 Purchase Agreement
+--- [START OF PAGE 2] ---
+TABLE OF CONTENTS
+     Page 
+ARTICLE I  DEFINITIONS AND USAGE   
+SECTION 1.1 Definitions    1 
+SECTION 1.2 Other Interpretive Provisions    1 
+ARTICLE II  PURCHASE   
+SECTION 2.1 Agreement to Sell and Contribute on the Closing Date    2 
+SECTION 2.2 Consideration and Payment for the Purchased Assets    2 
+ARTICLE III  REPRESENTATIONS, WARRANTIES AND COVENANTS   
+SECTION 3.1 Representations and Warranties of the Bank    2 
+SECTION 3.2 Representations and Warranties of the Bank Regarding the Purchased Assets    3 
+SECTION 3.3 Representations and Warranties of the Bank as to each Receivable    4 
+SECTION 3.4 Repurchase upon Breach    4 
+SECTION 3.5 Protection of Title    5 
+SECTION 3.6 Other Liens or Interests    6 
+SECTION 3.7 Official Record    6 
+SECTION 3.8 Merger or Consolidation of, or Assumption of the Obligations of, the Bank    6 
+SECTION 3.9 Bank May Own Notes and Certificates    6 
+SECTION 3.10 Compliance with the FDIC Rule    7 
+SECTION 3.11 Dispute Resolution    7 
+SECTION 3.12 Cooperation with Voting    11 
+ARTICLE IV  MISCELLANEOUS   
+SECTION 4.1 Transfers Intended as Sale; Security Interest    11 
+SECTION 4.2 Notices, Etc.    12 
+SECTION 4.3 Choice of Law    12 
+SECTION 4.4 Headings    12 
+SECTION 4.5 Counterparts    12 
+SECTION 4.6 Amendment    12 
+SECTION 4.7 Waivers    14 
+SECTION 4.8 Entire Agreement    14 
+  -i-   COPAR 2023-1 Purchase Agreement
+--- [START OF PAGE 3] ---
+TABLE OF CONTENTS
+(continued)
+     Page 
+SECTION 4.9 Severability of Provisions    14 
+SECTION 4.10 Binding Effect    14 
+SECTION 4.11 Acknowledgment and Agreement    14 
+SECTION 4.12 Cumulative Remedies    14 
+SECTION 4.13 Nonpetition Covenant    14 
+SECTION 4.14 Submission to Jurisdiction; Waiver of Jury Trial    15 
+SECTION 4.15 Not Applicable to the Bank in Other Capacities    15 
+SECTION 4.16 Third-Party Beneficiaries    15 
+EXHIBITS
+Exhibit A  Form of Assignment Pursuant to Purchase Agreement
+Schedule I  Perfection Representations, Warranties and Covenants
+Schedule II  Representations and Warranties with Respect to the Receivables
+  -ii-   COPAR 2023-1 Purchase Agreement
+--- [START OF PAGE 4] ---
+THIS PURCHASE AGREEMENT is made and entered into as of February 23, 2023 (as amended, restated, supplemented or otherwise modified
+and in effect from time to time, this “Agreement”) by CAPITAL ONE, NATIONAL ASSOCIATION, a national banking association (the “Bank”), and
+CAPITAL ONE AUTO RECEIVABLES, LLC, a Delaware limited liability company (“COAR”).
+WITNESSETH:
+WHEREAS, COAR desires to purchase from the Bank a portfolio of motor vehicle receivables, including motor vehicle retail installment sale
+contracts and/or installment loans that are secured by new and used automobiles, light-duty trucks, SUVs and vans; and
+WHEREAS, the Bank is willing to sell such portfolio of motor vehicle receivables and related property to COAR on the terms and conditions set
+forth in this Agreement.
+NOW, THEREFORE, in consideration of the premises and the mutual agreements set forth herein, the parties hereto agree as follows:
+ARTICLE I
+DEFINITIONS AND USAGE
+SECTION 1.1Definitions. Except as otherwise defined herein or as the context may otherwise require, capitalized terms used but not
+otherwise defined herein are defined in Appendix A to the Sale Agreement, dated as of the date hereof (as amended, supplemented, or otherwise
+modified and in effect from time to time, the “Sale Agreement”), between the Issuer and COAR, which also contains rules as to usage that are applicable
+herein. As used herein, the following terms shall have the following meanings:
+“Purchased Assets” has the meaning specified in Section 2.1.
+SECTION 1.2Other Interpretive Provisions. For purposes of this Agreement, unless the context otherwise requires: (a) accounting terms
+not otherwise defined in this Agreement, and accounting terms partly defined in this Agreement to the extent not defined, shall have the respective
+meanings given to them under GAAP (provided, that, to the extent that the definitions in this Agreement and GAAP conflict, the definitions in this
+Agreement shall control); (b) terms defined in Article 9 of the UCC as in effect in the relevant jurisdiction and not otherwise defined in this Agreement
+are used as defined in that Article; (c) the words “hereof,” “herein” and “hereunder” and words of similar import refer to this Agreement as a whole and
+not to any particular provision of this Agreement; (d) references to any Article, Section, Schedule, Appendix or Exhibit are references to Articles,
+Sections, Schedules, Appendices and Exhibits in or to this Agreement and references to any paragraph, subsection, clause or other subdivision within
+any Section or definition refer to such paragraph, subsection, clause or other subdivision of such Section or definition; (e) the term “including” and all
+variations thereof means “including without limitation”; (f) except as otherwise expressly provided herein, references to any law or regulation refer to
+that law or regulation as amended from time to time and include any successor law or regulation; (g) references to any Person include that Person’s
+successors and assigns; and (h) headings are for purposes of reference only and shall not otherwise affect the meaning or interpretation of any provision
+hereof.
+COPAR 2023-1 Purchase Agreement
+--- [START OF PAGE 5] ---
+ARTICLE II
+PURCHASE
+SECTION 2.1Agreement to Sell and Contribute on the Closing Date. On the terms and subject to the conditions set forth in this
+Agreement, the Bank does hereby sell, transfer, assign, set over, contribute and otherwise convey to COAR without recourse (subject to the obligations
+herein) on the Closing Date all of its right, title, interest, claims and demands in, to and under the Receivables, the Collections after the Cut-Off Date,
+the Receivable Files and the Related Security relating thereto, whether now owned or hereafter acquired, as evidenced by an assignment substantially in
+the form of Exhibit A (the “Assignment”) delivered on the Closing Date (collectively, the “Purchased Assets”). The sale, transfer, assignment,
+contribution and conveyance made hereunder does not constitute and is not intended to result in an assumption by COAR of any obligation of the Bank
+to the Obligors, the Dealers, insurers or any other Person in connection with the Receivables or the other assets and properties conveyed hereunder or
+any agreement, document or instrument related thereto.
+SECTION 2.2Consideration and Payment for the Purchased Assets. The purchase price for the sale of the Purchased Assets sold to COAR
+on the Closing Date shall equal the estimated fair market value of the Purchased Assets on the Closing Date. Such purchase price shall be paid (a) in
+cash to the Bank in an amount agreed to between the Bank and COAR, (b) by delivery to or upon the order of CONA, the 144A Notes and, (c) to the
+extent not paid in cash by COAR, shall be paid by a capital contribution by the Bank of an undivided interest in such Purchased Assets that increases its
+equity interest in COAR in an amount equal to the excess of the estimated fair market value of the Purchased Assets over the amount of cash paid by
+COAR to the Bank and the value of the 144A Notes.
+ARTICLE III
+REPRESENTATIONS, WARRANTIES AND COVENANTS
+SECTION 3.1Representations and Warranties of the Bank. The Bank makes the following representations and warranties as of the Closing
+Date, on which COAR will be deemed to have relied in acquiring the Purchased Assets. The representations and warranties will survive the conveyance
+of the Purchased Assets to COAR pursuant to this Agreement, the conveyance of the Purchased Assets by COAR to the Issuer pursuant to the Sale
+Agreement and the Grant thereof by the Issuer to the Indenture Trustee for the benefit of the Noteholders pursuant to the Indenture.
+(a) Existence and Power. The Bank is a national banking association validly subsisting under the laws of the United States of America and
+has, in all material respects, all power and authority to carry on its business as it is now conducted. The Bank has obtained all necessary licenses and
+approvals in each jurisdiction where the failure to do so would materially and adversely affect the ability of the Bank to perform its obligations under
+this Agreement or affect the enforceability or collectability of the Receivables or any other part of the Purchased Assets.
+COPAR 2023-1 Purchase Agreement
+-2-
+--- [START OF PAGE 6] ---
+(b) Authorization and No Contravention. The execution, delivery and performance by the Bank of this Agreement (i) have been duly
+authorized by all necessary action on the part of the Bank and (ii) do not contravene or constitute a default under (A) any applicable order, law, rule or
+regulation, (B) its organizational documents or (C) any material agreement, contract, order or other instrument to which it is a party or its property is
+subject (other than violations which do not affect the legality, validity or enforceability of such agreements or which, individually or in the aggregate,
+would not materially and adversely affect the transactions contemplated by, or the Bank’s ability to perform its obligations under, this Agreement).
+(c) No Consent Required. No approval or authorization by, or filing with, any Governmental Authority is required in connection with the
+execution, delivery and performance by the Bank of this Agreement other than (i) UCC filings, (ii) approvals and authorizations that have previously
+been obtained and filings that have previously been made and (iii) approvals, authorizations or filings which, if not obtained or made, would not have a
+material adverse effect on the enforceability or collectability of the Receivables or any other part of the Purchased Assets or would not materially and
+adversely affect the ability of the Bank to perform its obligations under this Agreement.
+(d) Binding Effect. This Agreement constitutes the legal, valid and binding obligation of the Bank enforceable against the Bank in
+accordance with its terms, except as such enforceability may be limited by applicable bankruptcy, insolvency, reorganization, moratorium, receivership,
+conservatorship or other similar laws affecting the enforcement of creditors’ rights generally and, if applicable, the rights of creditors of banking
+corporations from time to time in effect or by general principles of equity.
+(e) No Proceedings. There are no Proceedings pending or, to the knowledge of the Bank, threatened against the Bank before or by any
+Governmental Authority that (i) assert the invalidity or unenforceability of this Agreement or (ii) seek any determination or ruling that would materially
+and adversely affect the performance by the Bank of its obligations under this Agreement.
+(f) Lien Filings. The Bank is not aware of any material judgment, ERISA or tax lien filings against the Bank.
+SECTION 3.2Representations and Warranties of the Bank Regarding the Purchased Assets. On the date hereof, the Bank hereby makes the
+following representations and warranties to COAR as to the Receivables sold, transferred, assigned, contributed and otherwise conveyed to COAR
+under this Agreement on which such representations and warranties COAR will be deemed to have relied in acquiring the Receivables and which will
+survive the conveyance of the Purchased Assets to COAR pursuant to this Agreement, the conveyance of the Purchased Assets by COAR to the Issuer
+pursuant to the Sale Agreement and the Grant thereof by the Issuer to the Indenture Trustee for the benefit of the Noteholders pursuant to the Indenture:
+(a) The Receivables were selected using selection procedures that were not known or intended by the Bank to be adverse to the Issuer.
+(b) The Receivables and the other Purchased Assets have been validly assigned by the Bank to COAR.
+COPAR 2023-1 Purchase Agreement
+-3-
+--- [START OF PAGE 7] ---
+(c) The information with respect to the Receivables transferred on the Closing Date as set forth in the Schedule of Receivables was true
+and correct in all material respects as of the Cut-Off Date.
+(d) No Receivables are pledged, assigned, sold, subject to a security interest or otherwise conveyed by the Bank other than pursuant to the
+Transaction Documents. The Bank has not authorized the filing of and is not aware of any financing statements against the Bank that includes a
+description of collateral covering any Receivable other than any financing statement relating to security interests granted under the Transaction
+Documents or that have been or, prior to the assignment of such Receivables hereunder, will be terminated, amended or released. This Agreement
+creates a valid and continuing security interest in the Receivables (other than the Related Security with respect thereto, to the extent that an ownership
+interest therein cannot be perfected by the filing of a financing statement) in favor of COAR which security interest is prior to all other Liens created by
+the Bank (other than Permitted Liens) with respect to the Receivables and is enforceable as such against all other creditors of and purchasers and
+assignees from the Bank.
+(e) The representations and warranties regarding creation, perfection and priority of security interests in the Purchased Assets, which are
+attached to this Agreement as Schedule I, are true and correct.
+SECTION 3.3Representations and Warranties of the Bank as to each Receivable. The Bank hereby makes the representations and
+warranties set forth on Schedule II as to the Receivables sold, transferred, assigned, set over and otherwise conveyed to COAR under this Agreement on
+which such representations and warranties COAR relies in acquiring the Receivables. Such representations and warranties shall survive the sale of the
+Purchased Assets by COAR to the Issuer under the Sale Agreement and the Grant of the Purchased Assets by the Issuer to the Indenture Trustee for the
+benefit of the Noteholders pursuant to the Indenture. Notwithstanding any statement to the contrary contained herein or in any other Transaction
+Document, the Bank shall not be required to notify any insurer with respect to any Insurance Policy obtained by an Obligor or to notify any Dealer about
+any aspect of the transaction contemplated by this Agreement. The Bank hereby agrees that the Issuer shall have the right to enforce any and all rights
+under this Agreement assigned to the Issuer under the Sale Agreement, including the right to cause the Bank to repurchase any Receivable with respect
+to which it is in breach of any of its representations and warranties set forth in Schedule II, directly against the Bank as though the Issuer were a party to
+this Agreement, and the Issuer shall not be obligated to exercise any such rights indirectly through COAR.
+SECTION 3.4Repurchase upon Breach. Upon discovery by or notice to a Responsible Officer of COAR or the Bank of a breach of any of
+the representations and warranties set forth in Section 3.3 with respect to any Receivable at the time such representations and warranties were made
+which materially and adversely affects the interests of the Issuer, the Noteholders or the Certificateholders, the party discovering such breach or
+receiving such notice shall give prompt written notice thereof to the other party; provided, that delivery of a Servicer’s Report which identifies that
+Receivables are being or have been repurchased shall be deemed to constitute prompt notice of such breach; provided, further, that the failure to give
+such notice shall not affect any obligation of the Bank hereunder. If the breach materially and adversely affects the
+COPAR 2023-1 Purchase Agreement
+-4-
+--- [START OF PAGE 8] ---
+interests of the Issuer, the Noteholders or the Certificateholders, then the Bank shall either (a) correct or cure such breach or (b) repurchase such
+Receivable from COAR (or its assignee), in either case on or before the Payment Date following the end of the Collection Period which includes the
+sixtieth (60th) day (or, if the Bank elects, an earlier date) after the date that the Bank became aware or was notified of such breach. Any such breach or
+failure will be deemed not to have a material and adverse effect if such breach or failure has not affected the ability of COAR (or its assignee) to receive
+and retain timely payment in full on such Receivable. Any such purchase by the Bank shall be at a price equal to the related Repurchase Price. In
+consideration for such repurchase, the Bank shall make (or shall cause to be made) a payment to COAR (or its assignee) equal to the Repurchase Price
+by depositing such amount into the Collection Account prior to noon, New York City time, on the date of such repurchase, if such repurchase date is not
+a Payment Date or, if such repurchase date is a Payment Date, then prior to the close of business on the Business Day prior to such repurchase date.
+Upon payment of such Repurchase Price by the Bank, COAR (or its assignee) shall release and shall execute and deliver such instruments of release,
+transfer or assignment, in each case without recourse or representation, as may be reasonably requested by the Bank to evidence such release, transfer or
+assignment or more effectively vest in the Bank or its designee any Receivable and the related Purchased Assets repurchased pursuant hereto. It is
+understood and agreed that the obligation of the Bank to purchase any Receivable as described above shall constitute the sole remedy respecting such
+breach available to COAR (or its assignee).
+SECTION 3.5Protection of Title.
+(a) The Bank shall authorize and file such financing statements and cause to be authorized and filed such continuation and other financing
+statements, all in such manner and in such places as may be required by law fully to preserve, maintain and protect the interest of COAR under this
+Agreement in the Purchased Assets (to the extent that the interest of COAR therein can be perfected by the filing of a financing statement). The Bank
+shall deliver (or cause to be delivered) to COAR file-stamped copies of, or filing receipts for, any document filed as provided above, as soon as available
+following such filing.
+(b) The Bank shall notify COAR in writing within ten (10) days following the occurrence of (i) any change in the Bank’s organizational
+structure as a banking corporation, (ii) any change in the Bank’s “location” (within the meaning of Section 9-307 of the UCC) and (iii) any change in the
+Bank’s name, and shall take all action prior to making such change (or shall have made arrangements to take such action substantially simultaneously
+with such change, if it is not practicable to take such action in advance) reasonably necessary or advisable in the opinion of COAR to amend all
+previously filed financing statements or continuation statements described in paragraph (a) above. The Bank will at all times maintain its “location”
+within the United States.
+(c) The Bank shall maintain (or shall cause the Servicer to maintain) its computer systems so that, from time to time after the conveyance
+under this Agreement of the Receivables, the master computer records (including any backup archives) that refer to a Receivable shall indicate clearly
+the interest of COAR (or any subsequent assignee of COAR) in such Receivable and that such Receivable is owned by such Person. Indication of such
+Person’s interest in a Receivable shall not be deleted from or modified on such computer systems until, and only until, the related Receivable shall have
+been paid in full or repurchased.
+COPAR 2023-1 Purchase Agreement
+-5-
+--- [START OF PAGE 9] ---
+(d) If at any time the Bank shall propose to sell, grant a security interest in or otherwise transfer any interest in motor vehicle receivables to
+any prospective purchaser, lender or other transferee, the Bank shall give to such prospective purchaser, lender or other transferee computer tapes,
+records or printouts (including any restored from backup archives) that, if they shall refer in any manner whatsoever to any Receivable, shall indicate
+clearly that such Receivable has been sold and is owned by COAR (or any subsequent assignee of COAR).
+SECTION 3.6Other Liens or Interests. Except for the conveyances and grants of security interests pursuant to this Agreement and the
+other Transaction Documents, the Bank shall not sell, pledge, assign or transfer the Receivables or other property transferred to COAR to any other
+Person, or grant, create, incur, assume or suffer to exist any Lien (other than Permitted Liens) on any interest therein, and the Bank shall defend the
+right, title and interest of COAR in, to and under such Receivables or other property transferred to COAR against all claims of third parties claiming
+through or under the Bank.
+SECTION 3.7Official Record. So long as the Notes and the Certificates remain outstanding, this Agreement shall be treated as an official
+record of the Bank within the meaning of Section 13(e) of the Federal Deposit Insurance Act (12 U.S.C. Section 1823(e)).
+SECTION 3.8Merger or Consolidation of, or Assumption of the Obligations of, the Bank. Any Person (i) into which the Bank may be
+merged or converted or with which it may be consolidated, to which it may sell or transfer its business and assets as a whole or substantially as a whole,
+(ii) resulting from any merger, sale, transfer, conversion, or consolidation to which the Bank shall be a party, (iii) succeeding to the business of the Bank,
+or (iv) more than 50% of the voting stock or voting power and 50% or more of the economic equity of which is owned directly or indirectly by Capital
+One Financial Corporation, which Person in any of the foregoing cases executes an agreement of assumption to perform every obligation of the Bank
+under this Agreement, will be the successor to the Bank under this Agreement without the execution or filing of any document or any further act on the
+part of any of the parties to this Agreement anything herein to the contrary notwithstanding. Notwithstanding the foregoing, if the Bank enters into any
+of the foregoing transactions and is not the surviving entity, the Bank will deliver to the Indenture Trustee and the Owner Trustee an Opinion of Counsel
+either (A) stating that, in the opinion of such counsel, all financing statements and continuation statements and amendments thereto have been executed
+and filed that are necessary to preserve and protect the interest of the Issuer and, if the Notes are Outstanding, the Indenture Trustee for the benefit of the
+Noteholders, respectively, in the Receivables, or (B) stating that, in the opinion of such counsel, no such action is necessary to preserve and protect such
+interest.
+SECTION 3.9Bank May Own Notes and Certificates. The Bank, and any Affiliate of the Bank, may in its individual or any other capacity
+become the owner or pledgee of Notes and Certificates with the same rights as it would have if it were not the Bank or an Affiliate thereof, except as
+otherwise expressly provided herein or in the other Transaction Documents. Except as set forth herein or in the other Transaction Documents, Notes and
+Certificates so owned by the Bank or any such Affiliate will have an equal and proportionate benefit under the provisions of this Agreement and the
+other Transaction Documents, without preference, priority, or distinction as among all of the Notes and Certificates.
+COPAR 2023-1 Purchase Agreement
+-6-
+--- [START OF PAGE 10] ---
+SECTION 3.10Compliance with the FDIC Rule. The Bank (i) shall perform the covenants set forth in Article XII of the Indenture
+applicable to it and (ii) shall facilitate compliance with Article XII of the Indenture by the Capital One Parties.
+SECTION 3.11Dispute Resolution.
+(a) If any Receivable is subject to repurchase pursuant to Section 3.4 of this Agreement, which repurchase is not resolved in accordance
+with the terms of this Agreement within one hundred eighty (180) days after notice is delivered to the Bank by a Requesting Investor, the Requesting
+Investor providing such notice (the “Requesting Party”) will have the right to refer the matter, at its discretion, to either third-party mediation (including
+nonbinding arbitration) or binding arbitration pursuant to this Section 3.11 and the Bank is hereby deemed to consent to the selected resolution method.
+At the end of the 180-day period described above, the Bank may provide notice informing the Requesting Party of the status of its request or, in the
+absence of any such notice, the Requesting Party may presume that its request remains unresolved. The Requesting Party must provide written notice of
+its intention to refer the matter to mediation (including nonbinding arbitration) or arbitration to the Bank within thirty (30) days following such 180th
+day. The Bank agrees to participate in the resolution method selected by the Requesting Party.
+(b) If the Requesting Party selects mediation (including nonbinding arbitration) as the resolution method, the following provisions will
+apply:
+(i) the mediation will be administered by the American Arbitration Association (the “AAA”) pursuant to its Commercial Arbitration
+Rules and Mediation Procedures in effect at the time the mediation is initiated (the “Rules”); provided, that if any of the provisions in the Rules
+are inconsistent with the procedures for the mediation or arbitration stated in this Agreement, the procedures in this Agreement will control;
+(ii) the mediator must be a Qualified Dispute Resolution Professional. Upon being supplied a list, by the AAA, of at least ten
+(10) potential mediators that are each Qualified Dispute Resolution Professionals, each of the Requesting Party and the Bank will have the right to
+exercise two (2) peremptory challenges within fourteen (14) days and to rank the remaining potential mediators in order of preference. The AAA
+will select the mediator from the remaining potential mediators on the list, respecting the preference choices of the parties to the extent possible;
+(iii) each of the Requesting Party and the Bank will use commercially reasonable efforts to begin the mediation within ten
+(10) Business Days of the selection of the mediator and to conclude the mediation within thirty (30) days of the start of the mediation;
+(iv) the fees and expenses of the mediation will be allocated as mutually agreed by the Requesting Party and the Bank as part of the
+mediation; and
+(v) a failure by the Requesting Party and the Bank to resolve a disputed matter through mediation shall not preclude either party from
+seeking a resolution of such matter through the initiation of a judicial proceeding in a court of competent jurisdiction, subject to Section 3.11(d)
+below.
+COPAR 2023-1 Purchase Agreement
+-7-
+--- [START OF PAGE 11] ---
+(c) If the Requesting Party selects arbitration as the resolution method, the following provisions will apply:
+(i) the arbitration will be held in accordance with the United States Arbitration Act, notwithstanding any choice of law provision in
+this Agreement, and under the auspices of the AAA and in accordance with the Rules;
+(ii) if the repurchase request specified in Section 3.11(a) involves the repurchase of an aggregate amount of Receivables with an
+aggregate Outstanding Principal Balance of less than five percent (5%) of the total Outstanding Principal Balance of the Receivables as of the date
+of such repurchase request, a single arbitrator will be used. That arbitrator must be a Qualified Dispute Resolution Professional. Upon being
+supplied a list of at least ten (10) potential arbitrators that are each Qualified Dispute Resolutions Professionals by the AAA, each of the
+Requesting Party and the Bank will have the right to exercise two (2) peremptory challenges within fourteen (14) days and to rank the remaining
+potential arbitrators in order of preference. The AAA will select the arbitrator from the remaining potential arbitrators on the list respecting the
+preference choices of the parties to the extent possible;
+(iii) if the repurchase request specified in Section 3.11(a) involves the repurchase of an aggregate amount of Receivables with an
+aggregate Outstanding Principal Balance equal to or in excess of five percent (5%) of the total Outstanding Principal Balance of the Receivables
+as of the date of such repurchase request, a three-arbitrator panel will be used. The arbitral panel will consist of three Qualified Dispute Resolution
+Professionals, (A) one to be appointed by the Requesting Party within five (5) Business Days of providing notice to the Bank of its selection of
+arbitration, (B) one to be appointed by the Bank within five (5) Business Days of the Requesting Party’s appointment of an arbitrator, and (C) the
+third, who will preside over the arbitral panel, to be chosen by the two party-appointed arbitrators within five (5) Business Days of the Bank’s
+appointment. If any party fails to appoint an arbitrator or the two party-appointed arbitrators fail to appoint the third within the relevant time
+periods, then the appointments will be made by the AAA pursuant to the Rules;
+(iv) each arbitrator selected for any arbitration will abide by the Code of Ethics for Arbitrators in Commercial Disputes in effect at
+the time the arbitration is initiated. Prior to accepting an appointment, each arbitrator must promptly disclose any circumstances likely to create a
+reasonable inference of bias or conflict of interest or likely to preclude completion of the hearings within the prescribed time schedule. Any
+arbitrator selected may be removed by the AAA for cause consisting of actual bias, conflict of interest or other serious potential for conflict;
+COPAR 2023-1 Purchase Agreement
+-8-
+--- [START OF PAGE 12] ---
+(v) the Requesting Party and the Bank each agree that it is their intention that after consulting with the parties, the arbitrator or
+arbitral panel, as applicable, will devise procedures and deadlines for the arbitration, to the extent not already agreed to by the parties, with the
+goal of expediting the proceeding and completing the arbitration within thirty (30) days after appointment of the arbitrator or arbitral panel, as
+applicable. The arbitrator or the arbitral panel, as applicable, will have the authority to schedule, hear, and determine any and all motions,
+including dispositive and discovery motions, in accordance with New York law then in effect (including prehearing and post hearing motions), and
+will do so on the motion of any party to the arbitration. Notwithstanding any other discovery that may be available under the Rules, unless
+otherwise agreed by the parties, each party to the arbitration will be limited to the following discovery in the arbitration:
+(A) consistent with the expedited nature of arbitration, the Requesting Party and the Bank will, upon the written request of the other
+party, promptly provide the other with copies of documents relevant to the issues raised by any claim or counterclaim on which the
+producing party may rely in support of or in opposition to the claim or defense;
+(B) at the request of a party, the arbitrator or arbitral panel, as appl</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>{
+  "errors": [
+    {
+      "location": "Page 4, Section 1.1",
+      "error": "Incorporation-by-reference risk in a standalone fragment: key capitalized terms are defined only by reference to another document (Appendix A to the Sale Agreement), which is not included here. This leaves many deal-specific terms potentially undefined within this fragment.",
+      "suggestion": "Either (i) include Appendix A definitions in this document/append them, or (ii) expressly define in this Agreement each deal-specific term used herein (e.g., Issuer, Sale Agreement, Indenture, Noteholders, etc.) and attach any referenced schedules/appendices.",
+      "exact_quote": "capitalized terms used but not otherwise defined herein are defined in Appendix A to the Sale Agreement"
+    },
+    {
+      "location": "Page 5, Section 2.2",
+      "error": "Undefined unusual/deal-specific capitalized term: \"CONA\" is used but not defined in this fragment.",
+      "suggestion": "Define “CONA” in Section 1.1 (or replace with the full legal name of the applicable party).",
+      "exact_quote": "by delivery to or upon the order of CONA, the 144A Notes"
+    },
+    {
+      "location": "Page 5, Section 2.2",
+      "error": "Undefined unusual/deal-specific capitalized term: \"144A Notes\" is used but not defined in this fragment.",
+      "suggestion": "Add a definition of “144A Notes” (including issuer, series/class, and governing instrument) or cross-reference a defined term that is included in this fragment.",
+      "exact_quote": "the 144A Notes"
+    },
+    {
+      "location": "Page 5, Section 3.1 (survival sentence)",
+      "error": "Undefined unusual/deal-specific capitalized terms used without definitions in this fragment (beyond common lending terms): \"Issuer\", \"Indenture Trustee\", \"Noteholders\", and \"Indenture\".",
+      "suggestion": "Define each term in Section 1.1 or incorporate the relevant definitions directly into this Agreement (or attach the relevant definitional appendix).",
+      "exact_quote": "the conveyance of the Purchased Assets by COAR to the Issuer pursuant to the Sale Agreement and the Grant thereof by the Issuer to the Indenture Trustee for the benefit of the Noteholders pursuant to the Indenture."
+    },
+    {
+      "location": "Page 7, Section 3.4",
+      "error": "Grammar/clarity issue: plural noun used where singular is intended (or missing article). \"identifies that Receivables\" should be \"identifies that Receivables are\" (if plural) or \"identifies a Receivable\" (if singular).",
+      "suggestion": "Revise to: \"identifies that Receivables are being or have been repurchased\" (add \"are\"), or change \"Receivables\" to \"a Receivable\" as appropriate.",
+      "exact_quote": "a Servicer’s Report which identifies that\nReceivables are being or have been repurchased"
+    },
+    {
+      "location": "Page 11, Section 3.11(c)(ii)",
+      "error": "Typographical error in defined phrase: \"Qualified Dispute Resolutions Professionals\" should be \"Qualified Dispute Resolution Professionals\" (singular 'Resolution').",
+      "suggestion": "Replace \"Qualified Dispute Resolutions Professionals\" with \"Qualified Dispute Resolution Professionals\".",
+      "exact_quote": "potential arbitrators that are each Qualified Dispute Resolutions Professionals"
+    },
+    {
+      "location": "Page 14, Section 3.12",
+      "error": "Undefined unusual/deal-specific capitalized term: \"Instituting Noteholders\" is used but not defined in this fragment.",
+      "suggestion": "Define “Instituting Noteholders” or replace with an already-defined term (e.g., “Noteholders”) with the intended threshold/meaning stated.",
+      "exact_quote": "facilitate any vote by the Instituting Noteholders"
+    },
+    {
+      "location": "Page 15, Section 4.2",
+      "error": "Internal cross-reference appears incorrect: Notice provisions refer to \"Schedule I to the Sale Agreement\" for email addresses, but in this Agreement \"Schedule I\" is a Perfection schedule to this Agreement and may create confusion in a standalone read.",
+      "suggestion": "Clarify by specifying “Schedule I (Notices) to the Sale Agreement” (if that is a separate notices schedule) or attach/replicate the notice details in this Agreement.",
+      "exact_quote": "by e-mail (if an applicable e-mail address\nis provided on Schedule I to the Sale Agreement)"
+    },
+    {
+      "location": "Page 17, Section 4.7",
+      "error": "Missing comma creates ambiguity in list of parties: \"COAR the Servicer\" should be \"COAR, the Servicer\".",
+      "suggestion": "Insert a comma after “COAR”.",
+      "exact_quote": "No failure or delay on the part of COAR the Servicer"
+    },
+    {
+      "location": "Page 22, Exhibit A (date line)",
+      "error": "Unfilled placeholder bracket for the assignment date.",
+      "suggestion": "Replace the bracketed blank with the correct date (e.g., \"[•]\", or the actual month/day), or revise to a fixed date consistent with the transaction.",
+      "exact_quote": "[_________], 2023"
+    },
+    {
+      "location": "Page 23, Exhibit A signature block",
+      "error": "Signature block contains blanks/unfinished fields (By/Name/Title).",
+      "suggestion": "Complete the signature block with the authorized signatory name and title and insert the signature line formatting as needed.",
+      "exact_quote": "By:  \nName:\nTitle:"
+    },
+    {
+      "location": "Page 24, Schedule I heading",
+      "error": "Duplicative heading: \"SCHEDULE I\" appears twice consecutively.",
+      "suggestion": "Delete one instance of \"SCHEDULE I\".",
+      "exact_quote": "SCHEDULE I\nSCHEDULE I"
+    },
+    {
+      "location": "Page 25, Schedule I, paragraph 7",
+      "error": "Potential structural inconsistency: Schedule I paragraph 7 addresses delivery/possession arrangements involving the \"Indenture Trustee\" and \"Issuer\" at a stage that may not align with this Bank-to-COAR purchase agreement (it reads like downstream pledge/custody mechanics). In a standalone fragment, this is logically confusing and may be misplaced or should be expressly tied to the intended transaction step/timing.",
+      "suggestion": "Clarify timing and applicability (e.g., \"as of the Closing Date\" or \"upon subsequent transfer to the Issuer\") or move these provisions to the Sale Agreement/Indenture-related document if that is where they belong.",
+      "exact_quote": "All original executed copies of each such instrument or tangible chattel paper have been delivered to the Indenture Trustee, as pledgee of the\nIssuer"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-03-03 21:31:49</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>gpt-5-nano-2025-08-07</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>dc95508e-ea25-4e78-a846-6cfc255ad0a6.pdf</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document f...</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document fragment.
+Input: The attached text from a contract.
+CRITICAL INSTRUCTIONS:
+1. **Assume Isolation with Common Sense**: Do NOT assume missing definitions exist in other documents. However, IGNORE common commercial lending terms typically defined in a base Credit Agreement (e.g., "Borrower", "Administrative Agent", "Lender", "Business Day", "Dollars", "GAAP", "Material Adverse Effect"). Only flag specific, deal-specific, or unusual capitalized terms that are undefined.
+2. **Logic Check:** Check all math and logic tables.
+3. **Drafting Errors:** Find any placeholders like "[__]" or blank lines that were forgotten.
+4. **Exact Quotes:** For every error, you MUST provide the `exact_quote` from the text that contains the error. This is used for highlighting.
+Output Format:
+Return ONLY a valid JSON object with the following structure:
+{
+  "errors": [
+    {
+      "location": "Page 3, Section 2.1",
+      "error": "Description of the error",
+      "suggestion": "Suggested fix",
+      "exact_quote": "Exact text substring to highlight in red"
+    }
+  ]
+}
+If no errors are found, return {"errors": []}.
+--- CONTRACT TEXT BEGINS ---
+--- [START OF PAGE 1] ---
+EX-10.1 4 d45101 1dex101.htm EX-10.1
+Exhibit 10.1
+PURCHASE AGREEMENT
+dated as of February 23, 2023
+between
+CAPITAL ONE, NATIONAL ASSOCIATION
+and
+CAPITAL ONE AUTO RECEIVABLES, LLC,
+as Purchaser
+COPAR 2023-1 Purchase Agreement
+--- [START OF PAGE 2] ---
+TABLE OF CONTENTS
+     Page 
+ARTICLE I  DEFINITIONS AND USAGE   
+SECTION 1.1 Definitions    1 
+SECTION 1.2 Other Interpretive Provisions    1 
+ARTICLE II  PURCHASE   
+SECTION 2.1 Agreement to Sell and Contribute on the Closing Date    2 
+SECTION 2.2 Consideration and Payment for the Purchased Assets    2 
+ARTICLE III  REPRESENTATIONS, WARRANTIES AND COVENANTS   
+SECTION 3.1 Representations and Warranties of the Bank    2 
+SECTION 3.2 Representations and Warranties of the Bank Regarding the Purchased Assets    3 
+SECTION 3.3 Representations and Warranties of the Bank as to each Receivable    4 
+SECTION 3.4 Repurchase upon Breach    4 
+SECTION 3.5 Protection of Title    5 
+SECTION 3.6 Other Liens or Interests    6 
+SECTION 3.7 Official Record    6 
+SECTION 3.8 Merger or Consolidation of, or Assumption of the Obligations of, the Bank    6 
+SECTION 3.9 Bank May Own Notes and Certificates    6 
+SECTION 3.10 Compliance with the FDIC Rule    7 
+SECTION 3.11 Dispute Resolution    7 
+SECTION 3.12 Cooperation with Voting    11 
+ARTICLE IV  MISCELLANEOUS   
+SECTION 4.1 Transfers Intended as Sale; Security Interest    11 
+SECTION 4.2 Notices, Etc.    12 
+SECTION 4.3 Choice of Law    12 
+SECTION 4.4 Headings    12 
+SECTION 4.5 Counterparts    12 
+SECTION 4.6 Amendment    12 
+SECTION 4.7 Waivers    14 
+SECTION 4.8 Entire Agreement    14 
+  -i-   COPAR 2023-1 Purchase Agreement
+--- [START OF PAGE 3] ---
+TABLE OF CONTENTS
+(continued)
+     Page 
+SECTION 4.9 Severability of Provisions    14 
+SECTION 4.10 Binding Effect    14 
+SECTION 4.11 Acknowledgment and Agreement    14 
+SECTION 4.12 Cumulative Remedies    14 
+SECTION 4.13 Nonpetition Covenant    14 
+SECTION 4.14 Submission to Jurisdiction; Waiver of Jury Trial    15 
+SECTION 4.15 Not Applicable to the Bank in Other Capacities    15 
+SECTION 4.16 Third-Party Beneficiaries    15 
+EXHIBITS
+Exhibit A  Form of Assignment Pursuant to Purchase Agreement
+Schedule I  Perfection Representations, Warranties and Covenants
+Schedule II  Representations and Warranties with Respect to the Receivables
+  -ii-   COPAR 2023-1 Purchase Agreement
+--- [START OF PAGE 4] ---
+THIS PURCHASE AGREEMENT is made and entered into as of February 23, 2023 (as amended, restated, supplemented or otherwise modified
+and in effect from time to time, this “Agreement”) by CAPITAL ONE, NATIONAL ASSOCIATION, a national banking association (the “Bank”), and
+CAPITAL ONE AUTO RECEIVABLES, LLC, a Delaware limited liability company (“COAR”).
+WITNESSETH:
+WHEREAS, COAR desires to purchase from the Bank a portfolio of motor vehicle receivables, including motor vehicle retail installment sale
+contracts and/or installment loans that are secured by new and used automobiles, light-duty trucks, SUVs and vans; and
+WHEREAS, the Bank is willing to sell such portfolio of motor vehicle receivables and related property to COAR on the terms and conditions set
+forth in this Agreement.
+NOW, THEREFORE, in consideration of the premises and the mutual agreements set forth herein, the parties hereto agree as follows:
+ARTICLE I
+DEFINITIONS AND USAGE
+SECTION 1.1Definitions. Except as otherwise defined herein or as the context may otherwise require, capitalized terms used but not
+otherwise defined herein are defined in Appendix A to the Sale Agreement, dated as of the date hereof (as amended, supplemented, or otherwise
+modified and in effect from time to time, the “Sale Agreement”), between the Issuer and COAR, which also contains rules as to usage that are applicable
+herein. As used herein, the following terms shall have the following meanings:
+“Purchased Assets” has the meaning specified in Section 2.1.
+SECTION 1.2Other Interpretive Provisions. For purposes of this Agreement, unless the context otherwise requires: (a) accounting terms
+not otherwise defined in this Agreement, and accounting terms partly defined in this Agreement to the extent not defined, shall have the respective
+meanings given to them under GAAP (provided, that, to the extent that the definitions in this Agreement and GAAP conflict, the definitions in this
+Agreement shall control); (b) terms defined in Article 9 of the UCC as in effect in the relevant jurisdiction and not otherwise defined in this Agreement
+are used as defined in that Article; (c) the words “hereof,” “herein” and “hereunder” and words of similar import refer to this Agreement as a whole and
+not to any particular provision of this Agreement; (d) references to any Article, Section, Schedule, Appendix or Exhibit are references to Articles,
+Sections, Schedules, Appendices and Exhibits in or to this Agreement and references to any paragraph, subsection, clause or other subdivision within
+any Section or definition refer to such paragraph, subsection, clause or other subdivision of such Section or definition; (e) the term “including” and all
+variations thereof means “including without limitation”; (f) except as otherwise expressly provided herein, references to any law or regulation refer to
+that law or regulation as amended from time to time and include any successor law or regulation; (g) references to any Person include that Person’s
+successors and assigns; and (h) headings are for purposes of reference only and shall not otherwise affect the meaning or interpretation of any provision
+hereof.
+COPAR 2023-1 Purchase Agreement
+--- [START OF PAGE 5] ---
+ARTICLE II
+PURCHASE
+SECTION 2.1Agreement to Sell and Contribute on the Closing Date. On the terms and subject to the conditions set forth in this
+Agreement, the Bank does hereby sell, transfer, assign, set over, contribute and otherwise convey to COAR without recourse (subject to the obligations
+herein) on the Closing Date all of its right, title, interest, claims and demands in, to and under the Receivables, the Collections after the Cut-Off Date,
+the Receivable Files and the Related Security relating thereto, whether now owned or hereafter acquired, as evidenced by an assignment substantially in
+the form of Exhibit A (the “Assignment”) delivered on the Closing Date (collectively, the “Purchased Assets”). The sale, transfer, assignment,
+contribution and conveyance made hereunder does not constitute and is not intended to result in an assumption by COAR of any obligation of the Bank
+to the Obligors, the Dealers, insurers or any other Person in connection with the Receivables or the other assets and properties conveyed hereunder or
+any agreement, document or instrument related thereto.
+SECTION 2.2Consideration and Payment for the Purchased Assets. The purchase price for the sale of the Purchased Assets sold to COAR
+on the Closing Date shall equal the estimated fair market value of the Purchased Assets on the Closing Date. Such purchase price shall be paid (a) in
+cash to the Bank in an amount agreed to between the Bank and COAR, (b) by delivery to or upon the order of CONA, the 144A Notes and, (c) to the
+extent not paid in cash by COAR, shall be paid by a capital contribution by the Bank of an undivided interest in such Purchased Assets that increases its
+equity interest in COAR in an amount equal to the excess of the estimated fair market value of the Purchased Assets over the amount of cash paid by
+COAR to the Bank and the value of the 144A Notes.
+ARTICLE III
+REPRESENTATIONS, WARRANTIES AND COVENANTS
+SECTION 3.1Representations and Warranties of the Bank. The Bank makes the following representations and warranties as of the Closing
+Date, on which COAR will be deemed to have relied in acquiring the Purchased Assets. The representations and warranties will survive the conveyance
+of the Purchased Assets to COAR pursuant to this Agreement, the conveyance of the Purchased Assets by COAR to the Issuer pursuant to the Sale
+Agreement and the Grant thereof by the Issuer to the Indenture Trustee for the benefit of the Noteholders pursuant to the Indenture.
+(a) Existence and Power. The Bank is a national banking association validly subsisting under the laws of the United States of America and
+has, in all material respects, all power and authority to carry on its business as it is now conducted. The Bank has obtained all necessary licenses and
+approvals in each jurisdiction where the failure to do so would materially and adversely affect the ability of the Bank to perform its obligations under
+this Agreement or affect the enforceability or collectability of the Receivables or any other part of the Purchased Assets.
+COPAR 2023-1 Purchase Agreement
+-2-
+--- [START OF PAGE 6] ---
+(b) Authorization and No Contravention. The execution, delivery and performance by the Bank of this Agreement (i) have been duly
+authorized by all necessary action on the part of the Bank and (ii) do not contravene or constitute a default under (A) any applicable order, law, rule or
+regulation, (B) its organizational documents or (C) any material agreement, contract, order or other instrument to which it is a party or its property is
+subject (other than violations which do not affect the legality, validity or enforceability of such agreements or which, individually or in the aggregate,
+would not materially and adversely affect the transactions contemplated by, or the Bank’s ability to perform its obligations under, this Agreement).
+(c) No Consent Required. No approval or authorization by, or filing with, any Governmental Authority is required in connection with the
+execution, delivery and performance by the Bank of this Agreement other than (i) UCC filings, (ii) approvals and authorizations that have previously
+been obtained and filings that have previously been made and (iii) approvals, authorizations or filings which, if not obtained or made, would not have a
+material adverse effect on the enforceability or collectability of the Receivables or any other part of the Purchased Assets or would not materially and
+adversely affect the ability of the Bank to perform its obligations under this Agreement.
+(d) Binding Effect. This Agreement constitutes the legal, valid and binding obligation of the Bank enforceable against the Bank in
+accordance with its terms, except as such enforceability may be limited by applicable bankruptcy, insolvency, reorganization, moratorium, receivership,
+conservatorship or other similar laws affecting the enforcement of creditors’ rights generally and, if applicable, the rights of creditors of banking
+corporations from time to time in effect or by general principles of equity.
+(e) No Proceedings. There are no Proceedings pending or, to the knowledge of the Bank, threatened against the Bank before or by any
+Governmental Authority that (i) assert the invalidity or unenforceability of this Agreement or (ii) seek any determination or ruling that would materially
+and adversely affect the performance by the Bank of its obligations under this Agreement.
+(f) Lien Filings. The Bank is not aware of any material judgment, ERISA or tax lien filings against the Bank.
+SECTION 3.2Representations and Warranties of the Bank Regarding the Purchased Assets. On the date hereof, the Bank hereby makes the
+following representations and warranties to COAR as to the Receivables sold, transferred, assigned, contributed and otherwise conveyed to COAR
+under this Agreement on which such representations and warranties COAR will be deemed to have relied in acquiring the Receivables and which will
+survive the conveyance of the Purchased Assets to COAR pursuant to this Agreement, the conveyance of the Purchased Assets by COAR to the Issuer
+pursuant to the Sale Agreement and the Grant thereof by the Issuer to the Indenture Trustee for the benefit of the Noteholders pursuant to the Indenture:
+(a) The Receivables were selected using selection procedures that were not known or intended by the Bank to be adverse to the Issuer.
+(b) The Receivables and the other Purchased Assets have been validly assigned by the Bank to COAR.
+COPAR 2023-1 Purchase Agreement
+-3-
+--- [START OF PAGE 7] ---
+(c) The information with respect to the Receivables transferred on the Closing Date as set forth in the Schedule of Receivables was true
+and correct in all material respects as of the Cut-Off Date.
+(d) No Receivables are pledged, assigned, sold, subject to a security interest or otherwise conveyed by the Bank other than pursuant to the
+Transaction Documents. The Bank has not authorized the filing of and is not aware of any financing statements against the Bank that includes a
+description of collateral covering any Receivable other than any financing statement relating to security interests granted under the Transaction
+Documents or that have been or, prior to the assignment of such Receivables hereunder, will be terminated, amended or released. This Agreement
+creates a valid and continuing security interest in the Receivables (other than the Related Security with respect thereto, to the extent that an ownership
+interest therein cannot be perfected by the filing of a financing statement) in favor of COAR which security interest is prior to all other Liens created by
+the Bank (other than Permitted Liens) with respect to the Receivables and is enforceable as such against all other creditors of and purchasers and
+assignees from the Bank.
+(e) The representations and warranties regarding creation, perfection and priority of security interests in the Purchased Assets, which are
+attached to this Agreement as Schedule I, are true and correct.
+SECTION 3.3Representations and Warranties of the Bank as to each Receivable. The Bank hereby makes the representations and
+warranties set forth on Schedule II as to the Receivables sold, transferred, assigned, set over and otherwise conveyed to COAR under this Agreement on
+which such representations and warranties COAR relies in acquiring the Receivables. Such representations and warranties shall survive the sale of the
+Purchased Assets by COAR to the Issuer under the Sale Agreement and the Grant of the Purchased Assets by the Issuer to the Indenture Trustee for the
+benefit of the Noteholders pursuant to the Indenture. Notwithstanding any statement to the contrary contained herein or in any other Transaction
+Document, the Bank shall not be required to notify any insurer with respect to any Insurance Policy obtained by an Obligor or to notify any Dealer about
+any aspect of the transaction contemplated by this Agreement. The Bank hereby agrees that the Issuer shall have the right to enforce any and all rights
+under this Agreement assigned to the Issuer under the Sale Agreement, including the right to cause the Bank to repurchase any Receivable with respect
+to which it is in breach of any of its representations and warranties set forth in Schedule II, directly against the Bank as though the Issuer were a party to
+this Agreement, and the Issuer shall not be obligated to exercise any such rights indirectly through COAR.
+SECTION 3.4Repurchase upon Breach. Upon discovery by or notice to a Responsible Officer of COAR or the Bank of a breach of any of
+the representations and warranties set forth in Section 3.3 with respect to any Receivable at the time such representations and warranties were made
+which materially and adversely affects the interests of the Issuer, the Noteholders or the Certificateholders, the party discovering such breach or
+receiving such notice shall give prompt written notice thereof to the other party; provided, that delivery of a Servicer’s Report which identifies that
+Receivables are being or have been repurchased shall be deemed to constitute prompt notice of such breach; provided, further, that the failure to give
+such notice shall not affect any obligation of the Bank hereunder. If the breach materially and adversely affects the
+COPAR 2023-1 Purchase Agreement
+-4-
+--- [START OF PAGE 8] ---
+interests of the Issuer, the Noteholders or the Certificateholders, then the Bank shall either (a) correct or cure such breach or (b) repurchase such
+Receivable from COAR (or its assignee), in either case on or before the Payment Date following the end of the Collection Period which includes the
+sixtieth (60th) day (or, if the Bank elects, an earlier date) after the date that the Bank became aware or was notified of such breach. Any such breach or
+failure will be deemed not to have a material and adverse effect if such breach or failure has not affected the ability of COAR (or its assignee) to receive
+and retain timely payment in full on such Receivable. Any such purchase by the Bank shall be at a price equal to the related Repurchase Price. In
+consideration for such repurchase, the Bank shall make (or shall cause to be made) a payment to COAR (or its assignee) equal to the Repurchase Price
+by depositing such amount into the Collection Account prior to noon, New York City time, on the date of such repurchase, if such repurchase date is not
+a Payment Date or, if such repurchase date is a Payment Date, then prior to the close of business on the Business Day prior to such repurchase date.
+Upon payment of such Repurchase Price by the Bank, COAR (or its assignee) shall release and shall execute and deliver such instruments of release,
+transfer or assignment, in each case without recourse or representation, as may be reasonably requested by the Bank to evidence such release, transfer or
+assignment or more effectively vest in the Bank or its designee any Receivable and the related Purchased Assets repurchased pursuant hereto. It is
+understood and agreed that the obligation of the Bank to purchase any Receivable as described above shall constitute the sole remedy respecting such
+breach available to COAR (or its assignee).
+SECTION 3.5Protection of Title.
+(a) The Bank shall authorize and file such financing statements and cause to be authorized and filed such continuation and other financing
+statements, all in such manner and in such places as may be required by law fully to preserve, maintain and protect the interest of COAR under this
+Agreement in the Purchased Assets (to the extent that the interest of COAR therein can be perfected by the filing of a financing statement). The Bank
+shall deliver (or cause to be delivered) to COAR file-stamped copies of, or filing receipts for, any document filed as provided above, as soon as available
+following such filing.
+(b) The Bank shall notify COAR in writing within ten (10) days following the occurrence of (i) any change in the Bank’s organizational
+structure as a banking corporation, (ii) any change in the Bank’s “location” (within the meaning of Section 9-307 of the UCC) and (iii) any change in the
+Bank’s name, and shall take all action prior to making such change (or shall have made arrangements to take such action substantially simultaneously
+with such change, if it is not practicable to take such action in advance) reasonably necessary or advisable in the opinion of COAR to amend all
+previously filed financing statements or continuation statements described in paragraph (a) above. The Bank will at all times maintain its “location”
+within the United States.
+(c) The Bank shall maintain (or shall cause the Servicer to maintain) its computer systems so that, from time to time after the conveyance
+under this Agreement of the Receivables, the master computer records (including any backup archives) that refer to a Receivable shall indicate clearly
+the interest of COAR (or any subsequent assignee of COAR) in such Receivable and that such Receivable is owned by such Person. Indication of such
+Person’s interest in a Receivable shall not be deleted from or modified on such computer systems until, and only until, the related Receivable shall have
+been paid in full or repurchased.
+COPAR 2023-1 Purchase Agreement
+-5-
+--- [START OF PAGE 9] ---
+(d) If at any time the Bank shall propose to sell, grant a security interest in or otherwise transfer any interest in motor vehicle receivables to
+any prospective purchaser, lender or other transferee, the Bank shall give to such prospective purchaser, lender or other transferee computer tapes,
+records or printouts (including any restored from backup archives) that, if they shall refer in any manner whatsoever to any Receivable, shall indicate
+clearly that such Receivable has been sold and is owned by COAR (or any subsequent assignee of COAR).
+SECTION 3.6Other Liens or Interests. Except for the conveyances and grants of security interests pursuant to this Agreement and the
+other Transaction Documents, the Bank shall not sell, pledge, assign or transfer the Receivables or other property transferred to COAR to any other
+Person, or grant, create, incur, assume or suffer to exist any Lien (other than Permitted Liens) on any interest therein, and the Bank shall defend the
+right, title and interest of COAR in, to and under such Receivables or other property transferred to COAR against all claims of third parties claiming
+through or under the Bank.
+SECTION 3.7Official Record. So long as the Notes and the Certificates remain outstanding, this Agreement shall be treated as an official
+record of the Bank within the meaning of Section 13(e) of the Federal Deposit Insurance Act (12 U.S.C. Section 1823(e)).
+SECTION 3.8Merger or Consolidation of, or Assumption of the Obligations of, the Bank. Any Person (i) into which the Bank may be
+merged or converted or with which it may be consolidated, to which it may sell or transfer its business and assets as a whole or substantially as a whole,
+(ii) resulting from any merger, sale, transfer, conversion, or consolidation to which the Bank shall be a party, (iii) succeeding to the business of the Bank,
+or (iv) more than 50% of the voting stock or voting power and 50% or more of the economic equity of which is owned directly or indirectly by Capital
+One Financial Corporation, which Person in any of the foregoing cases executes an agreement of assumption to perform every obligation of the Bank
+under this Agreement, will be the successor to the Bank under this Agreement without the execution or filing of any document or any further act on the
+part of any of the parties to this Agreement anything herein to the contrary notwithstanding. Notwithstanding the foregoing, if the Bank enters into any
+of the foregoing transactions and is not the surviving entity, the Bank will deliver to the Indenture Trustee and the Owner Trustee an Opinion of Counsel
+either (A) stating that, in the opinion of such counsel, all financing statements and continuation statements and amendments thereto have been executed
+and filed that are necessary to preserve and protect the interest of the Issuer and, if the Notes are Outstanding, the Indenture Trustee for the benefit of the
+Noteholders, respectively, in the Receivables, or (B) stating that, in the opinion of such counsel, no such action is necessary to preserve and protect such
+interest.
+SECTION 3.9Bank May Own Notes and Certificates. The Bank, and any Affiliate of the Bank, may in its individual or any other capacity
+become the owner or pledgee of Notes and Certificates with the same rights as it would have if it were not the Bank or an Affiliate thereof, except as
+otherwise expressly provided herein or in the other Transaction Documents. Except as set forth herein or in the other Transaction Documents, Notes and
+Certificates so owned by the Bank or any such Affiliate will have an equal and proportionate benefit under the provisions of this Agreement and the
+other Transaction Documents, without preference, priority, or distinction as among all of the Notes and Certificates.
+COPAR 2023-1 Purchase Agreement
+-6-
+--- [START OF PAGE 10] ---
+SECTION 3.10Compliance with the FDIC Rule. The Bank (i) shall perform the covenants set forth in Article XII of the Indenture
+applicable to it and (ii) shall facilitate compliance with Article XII of the Indenture by the Capital One Parties.
+SECTION 3.11Dispute Resolution.
+(a) If any Receivable is subject to repurchase pursuant to Section 3.4 of this Agreement, which repurchase is not resolved in accordance
+with the terms of this Agreement within one hundred eighty (180) days after notice is delivered to the Bank by a Requesting Investor, the Requesting
+Investor providing such notice (the “Requesting Party”) will have the right to refer the matter, at its discretion, to either third-party mediation (including
+nonbinding arbitration) or binding arbitration pursuant to this Section 3.11 and the Bank is hereby deemed to consent to the selected resolution method.
+At the end of the 180-day period described above, the Bank may provide notice informing the Requesting Party of the status of its request or, in the
+absence of any such notice, the Requesting Party may presume that its request remains unresolved. The Requesting Party must provide written notice of
+its intention to refer the matter to mediation (including nonbinding arbitration) or arbitration to the Bank within thirty (30) days following such 180th
+day. The Bank agrees to participate in the resolution method selected by the Requesting Party.
+(b) If the Requesting Party selects mediation (including nonbinding arbitration) as the resolution method, the following provisions will
+apply:
+(i) the mediation will be administered by the American Arbitration Association (the “AAA”) pursuant to its Commercial Arbitration
+Rules and Mediation Procedures in effect at the time the mediation is initiated (the “Rules”); provided, that if any of the provisions in the Rules
+are inconsistent with the procedures for the mediation or arbitration stated in this Agreement, the procedures in this Agreement will control;
+(ii) the mediator must be a Qualified Dispute Resolution Professional. Upon being supplied a list, by the AAA, of at least ten
+(10) potential mediators that are each Qualified Dispute Resolution Professionals, each of the Requesting Party and the Bank will have the right to
+exercise two (2) peremptory challenges within fourteen (14) days and to rank the remaining potential mediators in order of preference. The AAA
+will select the mediator from the remaining potential mediators on the list, respecting the preference choices of the parties to the extent possible;
+(iii) each of the Requesting Party and the Bank will use commercially reasonable efforts to begin the mediation within ten
+(10) Business Days of the selection of the mediator and to conclude the mediation within thirty (30) days of the start of the mediation;
+(iv) the fees and expenses of the mediation will be allocated as mutually agreed by the Requesting Party and the Bank as part of the
+mediation; and
+(v) a failure by the Requesting Party and the Bank to resolve a disputed matter through mediation shall not preclude either party from
+seeking a resolution of such matter through the initiation of a judicial proceeding in a court of competent jurisdiction, subject to Section 3.11(d)
+below.
+COPAR 2023-1 Purchase Agreement
+-7-
+--- [START OF PAGE 11] ---
+(c) If the Requesting Party selects arbitration as the resolution method, the following provisions will apply:
+(i) the arbitration will be held in accordance with the United States Arbitration Act, notwithstanding any choice of law provision in
+this Agreement, and under the auspices of the AAA and in accordance with the Rules;
+(ii) if the repurchase request specified in Section 3.11(a) involves the repurchase of an aggregate amount of Receivables with an
+aggregate Outstanding Principal Balance of less than five percent (5%) of the total Outstanding Principal Balance of the Receivables as of the date
+of such repurchase request, a single arbitrator will be used. That arbitrator must be a Qualified Dispute Resolution Professional. Upon being
+supplied a list of at least ten (10) potential arbitrators that are each Qualified Dispute Resolutions Professionals by the AAA, each of the
+Requesting Party and the Bank will have the right to exercise two (2) peremptory challenges within fourteen (14) days and to rank the remaining
+potential arbitrators in order of preference. The AAA will select the arbitrator from the remaining potential arbitrators on the list respecting the
+preference choices of the parties to the extent possible;
+(iii) if the repurchase request specified in Section 3.11(a) involves the repurchase of an aggregate amount of Receivables with an
+aggregate Outstanding Principal Balance equal to or in excess of five percent (5%) of the total Outstanding Principal Balance of the Receivables
+as of the date of such repurchase request, a three-arbitrator panel will be used. The arbitral panel will consist of three Qualified Dispute Resolution
+Professionals, (A) one to be appointed by the Requesting Party within five (5) Business Days of providing notice to the Bank of its selection of
+arbitration, (B) one to be appointed by the Bank within five (5) Business Days of the Requesting Party’s appointment of an arbitrator, and (C) the
+third, who will preside over the arbitral panel, to be chosen by the two party-appointed arbitrators within five (5) Business Days of the Bank’s
+appointment. If any party fails to appoint an arbitrator or the two party-appointed arbitrators fail to appoint the third within the relevant time
+periods, then the appointments will be made by the AAA pursuant to the Rules;
+(iv) each arbitrator selected for any arbitration will abide by the Code of Ethics for Arbitrators in Commercial Disputes in effect at
+the time the arbitration is initiated. Prior to accepting an appointment, each arbitrator must promptly disclose any circumstances likely to create a
+reasonable inference of bias or conflict of interest or likely to preclude completion of the hearings within the prescribed time schedule. Any
+arbitrator selected may be removed by the AAA for cause consisting of actual bias, conflict of interest or other serious potential for conflict;
+COPAR 2023-1 Purchase Agreement
+-8-
+--- [START OF PAGE 12] ---
+(v) the Requesting Party and the Bank each agree that it is their intention that after consulting with the parties, the arbitrator or
+arbitral panel, as applicable, will devise procedures and deadlines for the arbitration, to the extent not already agreed to by the parties, with the
+goal of expediting the proceeding and completing the arbitration within thirty (30) days after appointment of the arbitrator or arbitral panel, as
+applicable. The arbitrator or the arbitral panel, as applicable, will have the authority to schedule, hear, and determine any and all motions,
+including dispositive and discovery motions, in accordance with New York law then in effect (including prehearing and post hearing motions), and
+will do so on the motion of any party to the arbitration. Notwithstanding any other discovery that may be available under the Rules, unless
+otherwise agreed by the parties, each party to the arbitration will be limited to the following discovery in the arbitration:
+(A) consistent with the expedited nature of arbitration, the Requesting Party and the Bank will, upon the written request of the other
+party, promptly provide the other with copies of documents relevant to the issues raised by any claim or counterclaim on which the
+producing party may rely in support of or in opposition to the claim or defense;
+(B) at the request of a party, the arbitrator or arbitral panel, as appl</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>{
+  "errors": [
+    {
+      "location": "Page 22, Exhibit A",
+      "error": "Missing execution date for the assignment; placeholder date not filled.",
+      "suggestion": "Insert the actual execution date for the Assignment (e.g., 'February 23, 2023').",
+      "exact_quote": "[_________], 2023"
+    },
+    {
+      "location": "Page 5, Section 2.2",
+      "error": "Undefined term 'CONA' used when describing payment consideration.",
+      "suggestion": "Determine the intended payee (likely COAR or another party) and replace 'CONA' accordingly, or add a defined term if 'CONA' is correct.",
+      "exact_quote": "by delivery to or upon the order of CONA, the 144A Notes and"
+    },
+    {
+      "location": "Page 4, Section 3.12",
+      "error": "Undefined/ambiguous term 'Instituting Noteholders' used in Cooperation with Voting.",
+      "suggestion": "Clarify or replace with the correct term (e.g., 'Initiating Noteholders' or a defined term in the Indenture) and ensure consistency with the Indenture.",
+      "exact_quote": "to facilitate any vote by the Instituting Noteholders pursuant to the terms of Section 7.6 of the Indenture"
+    },
+    {
+      "location": "Page 5, Section 2.1",
+      "error": "Usage of 'Cut-Off Date' without a clear definition in the Definitions section of this fragment.",
+      "suggestion": "Define 'Cut-Off Date' in the Definitions (or within Schedule II) or provide its explicit meaning to avoid ambiguity.",
+      "exact_quote": "Collections after the Cut-Off Date"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03-03 21:35:25</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>gemini-3-flash-preview</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>187f6a07-a87b-4b36-97be-24c11025d131.pdf</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document f...</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Role: You are a strict, pedantic Legal Proofreader. You are reviewing a standalone legal document fragment.
+Input: The attached text from a contract.
+CRITICAL INSTRUCTIONS:
+1. **Assume Isolation with Common Sense**: Do NOT assume missing definitions exist in other documents. However, IGNORE common commercial lending terms typically defined in a base Credit Agreement (e.g., "Borrower", "Administrative Agent", "Lender", "Business Day", "Dollars", "GAAP", "Material Adverse Effect"). Only flag specific, deal-specific, or unusual capitalized terms that are undefined.
+2. **Logic Check:** Check all math and logic tables.
+3. **Drafting Errors:** Find any placeholders like "[__]" or blank lines that were forgotten.
+4. **Exact Quotes:** For every error, you MUST provide the `exact_quote` from the text that contains the error. This is used for highlighting.
+Output Format:
+Return ONLY a valid JSON object with the following structure:
+{
+  "errors": [
+    {
+      "location": "Page 3, Section 2.1",
+      "error": "Description of the error",
+      "suggestion": "Suggested fix",
+      "exact_quote": "Exact text substring to highlight in red"
+    }
+  ]
+}
+If no errors are found, return {"errors": []}.
+--- CONTRACT TEXT BEGINS ---
+--- [START OF PAGE 1] ---
+EX-10.1 4 d45101 1dex101.htm EX-10.1
+Exhibit 10.1
+PURCHASE AGREEMENT
+dated as of February 23, 2023
+between
+CAPITAL ONE, NATIONAL ASSOCIATION
+and
+CAPITAL ONE AUTO RECEIVABLES, LLC,
+as Purchaser
+COPAR 2023-1 Purchase Agreement
+--- [START OF PAGE 2] ---
+TABLE OF CONTENTS
+     Page 
+ARTICLE I  DEFINITIONS AND USAGE   
+SECTION 1.1 Definitions    1 
+SECTION 1.2 Other Interpretive Provisions    1 
+ARTICLE II  PURCHASE   
+SECTION 2.1 Agreement to Sell and Contribute on the Closing Date    2 
+SECTION 2.2 Consideration and Payment for the Purchased Assets    2 
+ARTICLE III  REPRESENTATIONS, WARRANTIES AND COVENANTS   
+SECTION 3.1 Representations and Warranties of the Bank    2 
+SECTION 3.2 Representations and Warranties of the Bank Regarding the Purchased Assets    3 
+SECTION 3.3 Representations and Warranties of the Bank as to each Receivable    4 
+SECTION 3.4 Repurchase upon Breach    4 
+SECTION 3.5 Protection of Title    5 
+SECTION 3.6 Other Liens or Interests    6 
+SECTION 3.7 Official Record    6 
+SECTION 3.8 Merger or Consolidation of, or Assumption of the Obligations of, the Bank    6 
+SECTION 3.9 Bank May Own Notes and Certificates    6 
+SECTION 3.10 Compliance with the FDIC Rule    7 
+SECTION 3.11 Dispute Resolution    7 
+SECTION 3.12 Cooperation with Voting    11 
+ARTICLE IV  MISCELLANEOUS   
+SECTION 4.1 Transfers Intended as Sale; Security Interest    11 
+SECTION 4.2 Notices, Etc.    12 
+SECTION 4.3 Choice of Law    12 
+SECTION 4.4 Headings    12 
+SECTION 4.5 Counterparts    12 
+SECTION 4.6 Amendment    12 
+SECTION 4.7 Waivers    14 
+SECTION 4.8 Entire Agreement    14 
+  -i-   COPAR 2023-1 Purchase Agreement
+--- [START OF PAGE 3] ---
+TABLE OF CONTENTS
+(continued)
+     Page 
+SECTION 4.9 Severability of Provisions    14 
+SECTION 4.10 Binding Effect    14 
+SECTION 4.11 Acknowledgment and Agreement    14 
+SECTION 4.12 Cumulative Remedies    14 
+SECTION 4.13 Nonpetition Covenant    14 
+SECTION 4.14 Submission to Jurisdiction; Waiver of Jury Trial    15 
+SECTION 4.15 Not Applicable to the Bank in Other Capacities    15 
+SECTION 4.16 Third-Party Beneficiaries    15 
+EXHIBITS
+Exhibit A  Form of Assignment Pursuant to Purchase Agreement
+Schedule I  Perfection Representations, Warranties and Covenants
+Schedule II  Representations and Warranties with Respect to the Receivables
+  -ii-   COPAR 2023-1 Purchase Agreement
+--- [START OF PAGE 4] ---
+THIS PURCHASE AGREEMENT is made and entered into as of February 23, 2023 (as amended, restated, supplemented or otherwise modified
+and in effect from time to time, this “Agreement”) by CAPITAL ONE, NATIONAL ASSOCIATION, a national banking association (the “Bank”), and
+CAPITAL ONE AUTO RECEIVABLES, LLC, a Delaware limited liability company (“COAR”).
+WITNESSETH:
+WHEREAS, COAR desires to purchase from the Bank a portfolio of motor vehicle receivables, including motor vehicle retail installment sale
+contracts and/or installment loans that are secured by new and used automobiles, light-duty trucks, SUVs and vans; and
+WHEREAS, the Bank is willing to sell such portfolio of motor vehicle receivables and related property to COAR on the terms and conditions set
+forth in this Agreement.
+NOW, THEREFORE, in consideration of the premises and the mutual agreements set forth herein, the parties hereto agree as follows:
+ARTICLE I
+DEFINITIONS AND USAGE
+SECTION 1.1Definitions. Except as otherwise defined herein or as the context may otherwise require, capitalized terms used but not
+otherwise defined herein are defined in Appendix A to the Sale Agreement, dated as of the date hereof (as amended, supplemented, or otherwise
+modified and in effect from time to time, the “Sale Agreement”), between the Issuer and COAR, which also contains rules as to usage that are applicable
+herein. As used herein, the following terms shall have the following meanings:
+“Purchased Assets” has the meaning specified in Section 2.1.
+SECTION 1.2Other Interpretive Provisions. For purposes of this Agreement, unless the context otherwise requires: (a) accounting terms
+not otherwise defined in this Agreement, and accounting terms partly defined in this Agreement to the extent not defined, shall have the respective
+meanings given to them under GAAP (provided, that, to the extent that the definitions in this Agreement and GAAP conflict, the definitions in this
+Agreement shall control); (b) terms defined in Article 9 of the UCC as in effect in the relevant jurisdiction and not otherwise defined in this Agreement
+are used as defined in that Article; (c) the words “hereof,” “herein” and “hereunder” and words of similar import refer to this Agreement as a whole and
+not to any particular provision of this Agreement; (d) references to any Article, Section, Schedule, Appendix or Exhibit are references to Articles,
+Sections, Schedules, Appendices and Exhibits in or to this Agreement and references to any paragraph, subsection, clause or other subdivision within
+any Section or definition refer to such paragraph, subsection, clause or other subdivision of such Section or definition; (e) the term “including” and all
+variations thereof means “including without limitation”; (f) except as otherwise expressly provided herein, references to any law or regulation refer to
+that law or regulation as amended from time to time and include any successor law or regulation; (g) references to any Person include that Person’s
+successors and assigns; and (h) headings are for purposes of reference only and shall not otherwise affect the meaning or interpretation of any provision
+hereof.
+COPAR 2023-1 Purchase Agreement
+--- [START OF PAGE 5] ---
+ARTICLE II
+PURCHASE
+SECTION 2.1Agreement to Sell and Contribute on the Closing Date. On the terms and subject to the conditions set forth in this
+Agreement, the Bank does hereby sell, transfer, assign, set over, contribute and otherwise convey to COAR without recourse (subject to the obligations
+herein) on the Closing Date all of its right, title, interest, claims and demands in, to and under the Receivables, the Collections after the Cut-Off Date,
+the Receivable Files and the Related Security relating thereto, whether now owned or hereafter acquired, as evidenced by an assignment substantially in
+the form of Exhibit A (the “Assignment”) delivered on the Closing Date (collectively, the “Purchased Assets”). The sale, transfer, assignment,
+contribution and conveyance made hereunder does not constitute and is not intended to result in an assumption by COAR of any obligation of the Bank
+to the Obligors, the Dealers, insurers or any other Person in connection with the Receivables or the other assets and properties conveyed hereunder or
+any agreement, document or instrument related thereto.
+SECTION 2.2Consideration and Payment for the Purchased Assets. The purchase price for the sale of the Purchased Assets sold to COAR
+on the Closing Date shall equal the estimated fair market value of the Purchased Assets on the Closing Date. Such purchase price shall be paid (a) in
+cash to the Bank in an amount agreed to between the Bank and COAR, (b) by delivery to or upon the order of CONA, the 144A Notes and, (c) to the
+extent not paid in cash by COAR, shall be paid by a capital contribution by the Bank of an undivided interest in such Purchased Assets that increases its
+equity interest in COAR in an amount equal to the excess of the estimated fair market value of the Purchased Assets over the amount of cash paid by
+COAR to the Bank and the value of the 144A Notes.
+ARTICLE III
+REPRESENTATIONS, WARRANTIES AND COVENANTS
+SECTION 3.1Representations and Warranties of the Bank. The Bank makes the following representations and warranties as of the Closing
+Date, on which COAR will be deemed to have relied in acquiring the Purchased Assets. The representations and warranties will survive the conveyance
+of the Purchased Assets to COAR pursuant to this Agreement, the conveyance of the Purchased Assets by COAR to the Issuer pursuant to the Sale
+Agreement and the Grant thereof by the Issuer to the Indenture Trustee for the benefit of the Noteholders pursuant to the Indenture.
+(a) Existence and Power. The Bank is a national banking association validly subsisting under the laws of the United States of America and
+has, in all material respects, all power and authority to carry on its business as it is now conducted. The Bank has obtained all necessary licenses and
+approvals in each jurisdiction where the failure to do so would materially and adversely affect the ability of the Bank to perform its obligations under
+this Agreement or affect the enforceability or collectability of the Receivables or any other part of the Purchased Assets.
+COPAR 2023-1 Purchase Agreement
+-2-
+--- [START OF PAGE 6] ---
+(b) Authorization and No Contravention. The execution, delivery and performance by the Bank of this Agreement (i) have been duly
+authorized by all necessary action on the part of the Bank and (ii) do not contravene or constitute a default under (A) any applicable order, law, rule or
+regulation, (B) its organizational documents or (C) any material agreement, contract, order or other instrument to which it is a party or its property is
+subject (other than violations which do not affect the legality, validity or enforceability of such agreements or which, individually or in the aggregate,
+would not materially and adversely affect the transactions contemplated by, or the Bank’s ability to perform its obligations under, this Agreement).
+(c) No Consent Required. No approval or authorization by, or filing with, any Governmental Authority is required in connection with the
+execution, delivery and performance by the Bank of this Agreement other than (i) UCC filings, (ii) approvals and authorizations that have previously
+been obtained and filings that have previously been made and (iii) approvals, authorizations or filings which, if not obtained or made, would not have a
+material adverse effect on the enforceability or collectability of the Receivables or any other part of the Purchased Assets or would not materially and
+adversely affect the ability of the Bank to perform its obligations under this Agreement.
+(d) Binding Effect. This Agreement constitutes the legal, valid and binding obligation of the Bank enforceable against the Bank in
+accordance with its terms, except as such enforceability may be limited by applicable bankruptcy, insolvency, reorganization, moratorium, receivership,
+conservatorship or other similar laws affecting the enforcement of creditors’ rights generally and, if applicable, the rights of creditors of banking
+corporations from time to time in effect or by general principles of equity.
+(e) No Proceedings. There are no Proceedings pending or, to the knowledge of the Bank, threatened against the Bank before or by any
+Governmental Authority that (i) assert the invalidity or unenforceability of this Agreement or (ii) seek any determination or ruling that would materially
+and adversely affect the performance by the Bank of its obligations under this Agreement.
+(f) Lien Filings. The Bank is not aware of any material judgment, ERISA or tax lien filings against the Bank.
+SECTION 3.2Representations and Warranties of the Bank Regarding the Purchased Assets. On the date hereof, the Bank hereby makes the
+following representations and warranties to COAR as to the Receivables sold, transferred, assigned, contributed and otherwise conveyed to COAR
+under this Agreement on which such representations and warranties COAR will be deemed to have relied in acquiring the Receivables and which will
+survive the conveyance of the Purchased Assets to COAR pursuant to this Agreement, the conveyance of the Purchased Assets by COAR to the Issuer
+pursuant to the Sale Agreement and the Grant thereof by the Issuer to the Indenture Trustee for the benefit of the Noteholders pursuant to the Indenture:
+(a) The Receivables were selected using selection procedures that were not known or intended by the Bank to be adverse to the Issuer.
+(b) The Receivables and the other Purchased Assets have been validly assigned by the Bank to COAR.
+COPAR 2023-1 Purchase Agreement
+-3-
+--- [START OF PAGE 7] ---
+(c) The information with respect to the Receivables transferred on the Closing Date as set forth in the Schedule of Receivables was true
+and correct in all material respects as of the Cut-Off Date.
+(d) No Receivables are pledged, assigned, sold, subject to a security interest or otherwise conveyed by the Bank other than pursuant to the
+Transaction Documents. The Bank has not authorized the filing of and is not aware of any financing statements against the Bank that includes a
+description of collateral covering any Receivable other than any financing statement relating to security interests granted under the Transaction
+Documents or that have been or, prior to the assignment of such Receivables hereunder, will be terminated, amended or released. This Agreement
+creates a valid and continuing security interest in the Receivables (other than the Related Security with respect thereto, to the extent that an ownership
+interest therein cannot be perfected by the filing of a financing statement) in favor of COAR which security interest is prior to all other Liens created by
+the Bank (other than Permitted Liens) with respect to the Receivables and is enforceable as such against all other creditors of and purchasers and
+assignees from the Bank.
+(e) The representations and warranties regarding creation, perfection and priority of security interests in the Purchased Assets, which are
+attached to this Agreement as Schedule I, are true and correct.
+SECTION 3.3Representations and Warranties of the Bank as to each Receivable. The Bank hereby makes the representations and
+warranties set forth on Schedule II as to the Receivables sold, transferred, assigned, set over and otherwise conveyed to COAR under this Agreement on
+which such representations and warranties COAR relies in acquiring the Receivables. Such representations and warranties shall survive the sale of the
+Purchased Assets by COAR to the Issuer under the Sale Agreement and the Grant of the Purchased Assets by the Issuer to the Indenture Trustee for the
+benefit of the Noteholders pursuant to the Indenture. Notwithstanding any statement to the contrary contained herein or in any other Transaction
+Document, the Bank shall not be required to notify any insurer with respect to any Insurance Policy obtained by an Obligor or to notify any Dealer about
+any aspect of the transaction contemplated by this Agreement. The Bank hereby agrees that the Issuer shall have the right to enforce any and all rights
+under this Agreement assigned to the Issuer under the Sale Agreement, including the right to cause the Bank to repurchase any Receivable with respect
+to which it is in breach of any of its representations and warranties set forth in Schedule II, directly against the Bank as though the Issuer were a party to
+this Agreement, and the Issuer shall not be obligated to exercise any such rights indirectly through COAR.
+SECTION 3.4Repurchase upon Breach. Upon discovery by or notice to a Responsible Officer of COAR or the Bank of a breach of any of
+the representations and warranties set forth in Section 3.3 with respect to any Receivable at the time such representations and warranties were made
+which materially and adversely affects the interests of the Issuer, the Noteholders or the Certificateholders, the party discovering such breach or
+receiving such notice shall give prompt written notice thereof to the other party; provided, that delivery of a Servicer’s Report which identifies that
+Receivables are being or have been repurchased shall be deemed to constitute prompt notice of such breach; provided, further, that the failure to give
+such notice shall not affect any obligation of the Bank hereunder. If the breach materially and adversely affects the
+COPAR 2023-1 Purchase Agreement
+-4-
+--- [START OF PAGE 8] ---
+interests of the Issuer, the Noteholders or the Certificateholders, then the Bank shall either (a) correct or cure such breach or (b) repurchase such
+Receivable from COAR (or its assignee), in either case on or before the Payment Date following the end of the Collection Period which includes the
+sixtieth (60th) day (or, if the Bank elects, an earlier date) after the date that the Bank became aware or was notified of such breach. Any such breach or
+failure will be deemed not to have a material and adverse effect if such breach or failure has not affected the ability of COAR (or its assignee) to receive
+and retain timely payment in full on such Receivable. Any such purchase by the Bank shall be at a price equal to the related Repurchase Price. In
+consideration for such repurchase, the Bank shall make (or shall cause to be made) a payment to COAR (or its assignee) equal to the Repurchase Price
+by depositing such amount into the Collection Account prior to noon, New York City time, on the date of such repurchase, if such repurchase date is not
+a Payment Date or, if such repurchase date is a Payment Date, then prior to the close of business on the Business Day prior to such repurchase date.
+Upon payment of such Repurchase Price by the Bank, COAR (or its assignee) shall release and shall execute and deliver such instruments of release,
+transfer or assignment, in each case without recourse or representation, as may be reasonably requested by the Bank to evidence such release, transfer or
+assignment or more effectively vest in the Bank or its designee any Receivable and the related Purchased Assets repurchased pursuant hereto. It is
+understood and agreed that the obligation of the Bank to purchase any Receivable as described above shall constitute the sole remedy respecting such
+breach available to COAR (or its assignee).
+SECTION 3.5Protection of Title.
+(a) The Bank shall authorize and file such financing statements and cause to be authorized and filed such continuation and other financing
+statements, all in such manner and in such places as may be required by law fully to preserve, maintain and protect the interest of COAR under this
+Agreement in the Purchased Assets (to the extent that the interest of COAR therein can be perfected by the filing of a financing statement). The Bank
+shall deliver (or cause to be delivered) to COAR file-stamped copies of, or filing receipts for, any document filed as provided above, as soon as available
+following such filing.
+(b) The Bank shall notify COAR in writing within ten (10) days following the occurrence of (i) any change in the Bank’s organizational
+structure as a banking corporation, (ii) any change in the Bank’s “location” (within the meaning of Section 9-307 of the UCC) and (iii) any change in the
+Bank’s name, and shall take all action prior to making such change (or shall have made arrangements to take such action substantially simultaneously
+with such change, if it is not practicable to take such action in advance) reasonably necessary or advisable in the opinion of COAR to amend all
+previously filed financing statements or continuation statements described in paragraph (a) above. The Bank will at all times maintain its “location”
+within the United States.
+(c) The Bank shall maintain (or shall cause the Servicer to maintain) its computer systems so that, from time to time after the conveyance
+under this Agreement of the Receivables, the master computer records (including any backup archives) that refer to a Receivable shall indicate clearly
+the interest of COAR (or any subsequent assignee of COAR) in such Receivable and that such Receivable is owned by such Person. Indication of such
+Person’s interest in a Receivable shall not be deleted from or modified on such computer systems until, and only until, the related Receivable shall have
+been paid in full or repurchased.
+COPAR 2023-1 Purchase Agreement
+-5-
+--- [START OF PAGE 9] ---
+(d) If at any time the Bank shall propose to sell, grant a security interest in or otherwise transfer any interest in motor vehicle receivables to
+any prospective purchaser, lender or other transferee, the Bank shall give to such prospective purchaser, lender or other transferee computer tapes,
+records or printouts (including any restored from backup archives) that, if they shall refer in any manner whatsoever to any Receivable, shall indicate
+clearly that such Receivable has been sold and is owned by COAR (or any subsequent assignee of COAR).
+SECTION 3.6Other Liens or Interests. Except for the conveyances and grants of security interests pursuant to this Agreement and the
+other Transaction Documents, the Bank shall not sell, pledge, assign or transfer the Receivables or other property transferred to COAR to any other
+Person, or grant, create, incur, assume or suffer to exist any Lien (other than Permitted Liens) on any interest therein, and the Bank shall defend the
+right, title and interest of COAR in, to and under such Receivables or other property transferred to COAR against all claims of third parties claiming
+through or under the Bank.
+SECTION 3.7Official Record. So long as the Notes and the Certificates remain outstanding, this Agreement shall be treated as an official
+record of the Bank within the meaning of Section 13(e) of the Federal Deposit Insurance Act (12 U.S.C. Section 1823(e)).
+SECTION 3.8Merger or Consolidation of, or Assumption of the Obligations of, the Bank. Any Person (i) into which the Bank may be
+merged or converted or with which it may be consolidated, to which it may sell or transfer its business and assets as a whole or substantially as a whole,
+(ii) resulting from any merger, sale, transfer, conversion, or consolidation to which the Bank shall be a party, (iii) succeeding to the business of the Bank,
+or (iv) more than 50% of the voting stock or voting power and 50% or more of the economic equity of which is owned directly or indirectly by Capital
+One Financial Corporation, which Person in any of the foregoing cases executes an agreement of assumption to perform every obligation of the Bank
+under this Agreement, will be the successor to the Bank under this Agreement without the execution or filing of any document or any further act on the
+part of any of the parties to this Agreement anything herein to the contrary notwithstanding. Notwithstanding the foregoing, if the Bank enters into any
+of the foregoing transactions and is not the surviving entity, the Bank will deliver to the Indenture Trustee and the Owner Trustee an Opinion of Counsel
+either (A) stating that, in the opinion of such counsel, all financing statements and continuation statements and amendments thereto have been executed
+and filed that are necessary to preserve and protect the interest of the Issuer and, if the Notes are Outstanding, the Indenture Trustee for the benefit of the
+Noteholders, respectively, in the Receivables, or (B) stating that, in the opinion of such counsel, no such action is necessary to preserve and protect such
+interest.
+SECTION 3.9Bank May Own Notes and Certificates. The Bank, and any Affiliate of the Bank, may in its individual or any other capacity
+become the owner or pledgee of Notes and Certificates with the same rights as it would have if it were not the Bank or an Affiliate thereof, except as
+otherwise expressly provided herein or in the other Transaction Documents. Except as set forth herein or in the other Transaction Documents, Notes and
+Certificates so owned by the Bank or any such Affiliate will have an equal and proportionate benefit under the provisions of this Agreement and the
+other Transaction Documents, without preference, priority, or distinction as among all of the Notes and Certificates.
+COPAR 2023-1 Purchase Agreement
+-6-
+--- [START OF PAGE 10] ---
+SECTION 3.10Compliance with the FDIC Rule. The Bank (i) shall perform the covenants set forth in Article XII of the Indenture
+applicable to it and (ii) shall facilitate compliance with Article XII of the Indenture by the Capital One Parties.
+SECTION 3.11Dispute Resolution.
+(a) If any Receivable is subject to repurchase pursuant to Section 3.4 of this Agreement, which repurchase is not resolved in accordance
+with the terms of this Agreement within one hundred eighty (180) days after notice is delivered to the Bank by a Requesting Investor, the Requesting
+Investor providing such notice (the “Requesting Party”) will have the right to refer the matter, at its discretion, to either third-party mediation (including
+nonbinding arbitration) or binding arbitration pursuant to this Section 3.11 and the Bank is hereby deemed to consent to the selected resolution method.
+At the end of the 180-day period described above, the Bank may provide notice informing the Requesting Party of the status of its request or, in the
+absence of any such notice, the Requesting Party may presume that its request remains unresolved. The Requesting Party must provide written notice of
+its intention to refer the matter to mediation (including nonbinding arbitration) or arbitration to the Bank within thirty (30) days following such 180th
+day. The Bank agrees to participate in the resolution method selected by the Requesting Party.
+(b) If the Requesting Party selects mediation (including nonbinding arbitration) as the resolution method, the following provisions will
+apply:
+(i) the mediation will be administered by the American Arbitration Association (the “AAA”) pursuant to its Commercial Arbitration
+Rules and Mediation Procedures in effect at the time the mediation is initiated (the “Rules”); provided, that if any of the provisions in the Rules
+are inconsistent with the procedures for the mediation or arbitration stated in this Agreement, the procedures in this Agreement will control;
+(ii) the mediator must be a Qualified Dispute Resolution Professional. Upon being supplied a list, by the AAA, of at least ten
+(10) potential mediators that are each Qualified Dispute Resolution Professionals, each of the Requesting Party and the Bank will have the right to
+exercise two (2) peremptory challenges within fourteen (14) days and to rank the remaining potential mediators in order of preference. The AAA
+will select the mediator from the remaining potential mediators on the list, respecting the preference choices of the parties to the extent possible;
+(iii) each of the Requesting Party and the Bank will use commercially reasonable efforts to begin the mediation within ten
+(10) Business Days of the selection of the mediator and to conclude the mediation within thirty (30) days of the start of the mediation;
+(iv) the fees and expenses of the mediation will be allocated as mutually agreed by the Requesting Party and the Bank as part of the
+mediation; and
+(v) a failure by the Requesting Party and the Bank to resolve a disputed matter through mediation shall not preclude either party from
+seeking a resolution of such matter through the initiation of a judicial proceeding in a court of competent jurisdiction, subject to Section 3.11(d)
+below.
+COPAR 2023-1 Purchase Agreement
+-7-
+--- [START OF PAGE 11] ---
+(c) If the Requesting Party selects arbitration as the resolution method, the following provisions will apply:
+(i) the arbitration will be held in accordance with the United States Arbitration Act, notwithstanding any choice of law provision in
+this Agreement, and under the auspices of the AAA and in accordance with the Rules;
+(ii) if the repurchase request specified in Section 3.11(a) involves the repurchase of an aggregate amount of Receivables with an
+aggregate Outstanding Principal Balance of less than five percent (5%) of the total Outstanding Principal Balance of the Receivables as of the date
+of such repurchase request, a single arbitrator will be used. That arbitrator must be a Qualified Dispute Resolution Professional. Upon being
+supplied a list of at least ten (10) potential arbitrators that are each Qualified Dispute Resolutions Professionals by the AAA, each of the
+Requesting Party and the Bank will have the right to exercise two (2) peremptory challenges within fourteen (14) days and to rank the remaining
+potential arbitrators in order of preference. The AAA will select the arbitrator from the remaining potential arbitrators on the list respecting the
+preference choices of the parties to the extent possible;
+(iii) if the repurchase request specified in Section 3.11(a) involves the repurchase of an aggregate amount of Receivables with an
+aggregate Outstanding Principal Balance equal to or in excess of five percent (5%) of the total Outstanding Principal Balance of the Receivables
+as of the date of such repurchase request, a three-arbitrator panel will be used. The arbitral panel will consist of three Qualified Dispute Resolution
+Professionals, (A) one to be appointed by the Requesting Party within five (5) Business Days of providing notice to the Bank of its selection of
+arbitration, (B) one to be appointed by the Bank within five (5) Business Days of the Requesting Party’s appointment of an arbitrator, and (C) the
+third, who will preside over the arbitral panel, to be chosen by the two party-appointed arbitrators within five (5) Business Days of the Bank’s
+appointment. If any party fails to appoint an arbitrator or the two party-appointed arbitrators fail to appoint the third within the relevant time
+periods, then the appointments will be made by the AAA pursuant to the Rules;
+(iv) each arbitrator selected for any arbitration will abide by the Code of Ethics for Arbitrators in Commercial Disputes in effect at
+the time the arbitration is initiated. Prior to accepting an appointment, each arbitrator must promptly disclose any circumstances likely to create a
+reasonable inference of bias or conflict of interest or likely to preclude completion of the hearings within the prescribed time schedule. Any
+arbitrator selected may be removed by the AAA for cause consisting of actual bias, conflict of interest or other serious potential for conflict;
+COPAR 2023-1 Purchase Agreement
+-8-
+--- [START OF PAGE 12] ---
+(v) the Requesting Party and the Bank each agree that it is their intention that after consulting with the parties, the arbitrator or
+arbitral panel, as applicable, will devise procedures and deadlines for the arbitration, to the extent not already agreed to by the parties, with the
+goal of expediting the proceeding and completing the arbitration within thirty (30) days after appointment of the arbitrator or arbitral panel, as
+applicable. The arbitrator or the arbitral panel, as applicable, will have the authority to schedule, hear, and determine any and all motions,
+including dispositive and discovery motions, in accordance with New York law then in effect (including prehearing and post hearing motions), and
+will do so on the motion of any party to the arbitration. Notwithstanding any other discovery that may be available under the Rules, unless
+otherwise agreed by the parties, each party to the arbitration will be limited to the following discovery in the arbitration:
+(A) consistent with the expedited nature of arbitration, the Requesting Party and the Bank will, upon the written request of the other
+party, promptly provide the other with copies of documents relevant to the issues raised by any claim or counterclaim on which the
+producing party may rely in support of or in opposition to the claim or defense;
+(B) at the request of a party, the arbitrator or arbitral panel, as appl</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>{
+  "errors": [
+    {
+      "location": "Page 5, Section 2.2",
+      "error": "The acronym 'CONA' is used without being defined as a party alias. The preamble defines Capital One, National Association as 'the Bank'.",
+      "suggestion": "Define 'CONA' in the preamble or change the reference to 'the Bank'.",
+      "exact_quote": "by delivery to or upon the order of CONA"
+    },
+    {
+      "location": "Page 5, Section 2.2",
+      "error": "The term '144A Notes' is undefined and deal-specific. While Section 1.1 incorporates Appendix A of the Sale Agreement, securities descriptions usually require local definition or explicit cross-reference when they form the consideration for the purchase price.",
+      "suggestion": "Define '144A Notes' or ensure they are listed in the specific definitions of Section 1.1.",
+      "exact_quote": "the 144A Notes and"
+    },
+    {
+      "location": "Page 12, Section 3.11(c)(v)",
+      "error": "Logical conflict in arbitration timelines. The text expresses an intention to complete the arbitration within 30 days, but clause (D) allows 60 days for discovery.",
+      "suggestion": "Reconcile the timelines (e.g., extend the completion goal to 90 days or reduce discovery to 15 days).",
+      "exact_quote": "completing the arbitration within thirty (30) days after appointment of the arbitrator or arbitral panel, as applicable."
+    },
+    {
+      "location": "Page 22, Exhibit A",
+      "error": "Bracketed placeholder for the date was not completed.",
+      "suggestion": "Fill in the specific date of the assignment.",
+      "exact_quote": "[_________], 2023"
+    },
+    {
+      "location": "Page 23, Exhibit A",
+      "error": "The signature block contains blank lines for the signatory's name and title.",
+      "suggestion": "Insert the authorized officer's name and title.",
+      "exact_quote": "By:  \r\nName:\r\nTitle:"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>